<commit_message>
Update Stripe checkout entry execution results
Co-authored-by: ShobhaAml <ShobhaAml@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
+++ b/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +41,12 @@
       <b val="1"/>
       <color rgb="009C5700"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00274E13"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +61,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -100,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -115,6 +124,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -482,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -550,7 +562,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
@@ -560,7 +572,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
@@ -580,7 +592,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
@@ -591,7 +603,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RUN-STR-20261021-001</t>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Latest executed section</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1. Stripe Checkout Entry and Plan Selection</t>
         </is>
       </c>
     </row>
@@ -1541,8 +1565,8 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
-    <col width="31" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="47" customWidth="1" min="11" max="11"/>
     <col width="55" customWidth="1" min="12" max="12"/>
     <col width="55" customWidth="1" min="13" max="13"/>
     <col width="55" customWidth="1" min="14" max="14"/>
@@ -1657,6 +1681,51 @@
           <t>User is redirected to Stripe Checkout on checkout.stripe.com.</t>
         </is>
       </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Annual no-ads - 30 EUR/year</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>Subscribe CTA is visible and clickable, but clicking it redirected to Xataka auth page (/xtra/anual-sin-anuncios), not checkout.stripe.com. Stripe Checkout was not reached; flow stopped at Xataka authentication wall before checkout.stripe.com.</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/d5630.webp; /tmp/computer-use/263da.webp; /tmp/computer-use/a5800.webp</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>Authentication gate prevents confirming direct Stripe Checkout redirect for visitor flow.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -1689,6 +1758,51 @@
           <t>PayPal remains available for existing subscribers; Stripe is available for new subscription checkout.</t>
         </is>
       </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Landing page plans</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Landing page shows payment text: Paga con tarjeta o PayPal, cancela cuando quieras.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/d5630.webp; /tmp/computer-use/716c1.webp</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>PayPal coexistence is visible on the landing page. Existing PayPal subscriber behavior was not exercised because valid subscriber credentials were unavailable.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1721,6 +1835,51 @@
           <t>Stripe Checkout order summary shows monthly plan name, monthly price and monthly billing frequency.</t>
         </is>
       </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Monthly - 2 EUR/month</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>Monthly plan can be selected. The flow redirects to /xtra/mensual-con-anuncios and shows the selected monthly subscription with 4 EUR crossed out and 2 EUR/month.</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/3a0ac.webp; /tmp/computer-use/716c1.webp; /tmp/computer-use/8b686.webp; /tmp/computer-use/24ce9.webp</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>Plan selection works before authentication. Stripe Checkout summary was not reached.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -1753,6 +1912,51 @@
           <t>Stripe Checkout order summary shows annual plan name, annual price and annual billing frequency.</t>
         </is>
       </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year; Annual no-ads - 30 EUR/year</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>Annual plans can be selected. The flow redirects to /xtra/anual-con-anuncios for 15 EUR/year and /xtra/anual-sin-anuncios for 30 EUR/year.</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/c1a65.webp; /tmp/computer-use/e219c.webp; /tmp/computer-use/105dd.webp; /tmp/computer-use/5d469.webp</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>Plan selection works before authentication. Stripe Checkout summary was not reached.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1785,6 +1989,51 @@
           <t>Each plan maps to the correct Stripe Price ID and displayed amount.</t>
         </is>
       </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Monthly and annual plans</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>Displayed prices match landing/auth page expectations: monthly 4 EUR crossed out to 2 EUR/month; annual 30 EUR crossed out to 15 EUR/year; annual no-ads 60 EUR crossed out to 30 EUR/year. Discount messaging states 50 percent discount while subscription remains active.</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/d5630.webp; /tmp/computer-use/716c1.webp; /tmp/computer-use/24ce9.webp; /tmp/computer-use/5d469.webp</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>Visible price mapping passed on Xataka pages. Stripe Price IDs/session summary could not be verified because checkout was not reached.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -1817,6 +2066,51 @@
           <t>Payment UI is hosted by Stripe; Xataka does not render or collect card fields locally.</t>
         </is>
       </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Unable to verify hosted checkout mode. All subscription attempts stayed on Xataka auth pages; checkout.stripe.com was not reached.</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp; /tmp/computer-use/a5800.webp</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>Needs valid verified account to proceed past auth and inspect the payment page.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1849,6 +2143,51 @@
           <t>Email field is pre-filled with logged-in user email.</t>
         </is>
       </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Attempted QA accounts: testi.n.g.2.4.aug@gmail.com; testing24au.g2.6@gmail.com. Both rejected by login form.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Both provided QA accounts were rejected with the message: Tu correo electronico o tu contrasena no son correctos. Logged-in Stripe Checkout email prefill could not be verified.</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/02011.webp; /tmp/computer-use/71a68.webp</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Provide a valid verified account to test email prefill.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -1881,6 +2220,51 @@
           <t>Checkout allows user to enter email or follows configured authentication flow.</t>
         </is>
       </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>Anonymous Stripe Checkout email field could not be observed because the flow stayed on Xataka authentication/registration before Stripe Checkout.</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>Checkout email behavior requires reaching Stripe Checkout.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1913,6 +2297,51 @@
           <t>Stripe Checkout summary shows plan name, price, billing frequency and trial period.</t>
         </is>
       </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>Stripe order summary with trial could not be observed. No trial messaging was visible on landing/auth pages.</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>Requires checkout access and a plan configured with active trial.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1945,6 +2374,51 @@
           <t>Stripe Checkout summary shows plan name, price and billing frequency without trial messaging.</t>
         </is>
       </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>Stripe order summary without trial could not be observed because Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Requires checkout access.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1977,6 +2451,51 @@
           <t>User returns to Xataka subscription page.</t>
         </is>
       </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>Cancel/back behavior from Stripe Checkout could not be tested because Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>Requires checkout access.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -2009,6 +2528,51 @@
           <t>User returns to Xataka success/welcome page.</t>
         </is>
       </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>4000056655665556; 2223003122003222 (not used)</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Successful checkout and welcome redirect could not be tested because Stripe Checkout was not reached. Cards 4000056655665556 and 2223003122003222 were not entered or submitted because Stripe Checkout was not reached and test/sandbox mode was not confirmed.</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>Payment submission requires verified account and confirmed Stripe test/sandbox checkout.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -2041,6 +2605,51 @@
           <t>Xataka account is associated with active Stripe subscription/customer.</t>
         </is>
       </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Account association after successful checkout could not be verified because checkout completion was not possible.</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Requires successful checkout completion.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -2071,6 +2680,51 @@
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>No duplicate subscription or duplicate activation is created.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate activation prevention could not be tested because no checkout success URL/session was created.</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>Requires completed checkout and success URL/session replay.</t>
         </is>
       </c>
     </row>
@@ -5360,7 +6014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5368,8 +6022,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="47" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
@@ -5625,6 +6279,874 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-001</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Annual no-ads - 30 EUR/year</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Opened /xtra; clicked Suscribete ahora CTA; observed redirect.</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Subscribe CTA is visible and clickable, but clicking it redirected to Xataka auth page (/xtra/anual-sin-anuncios), not checkout.stripe.com. Stripe Checkout was not reached; flow stopped at Xataka authentication wall before checkout.stripe.com.</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/d5630.webp; /tmp/computer-use/263da.webp; /tmp/computer-use/a5800.webp</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Authentication gate prevents confirming direct Stripe Checkout redirect for visitor flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-002</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Landing page plans</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Opened /xtra; inspected payment method text below subscription CTA.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Landing page shows payment text: Paga con tarjeta o PayPal, cancela cuando quieras.</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/d5630.webp; /tmp/computer-use/716c1.webp</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>PayPal coexistence is visible on the landing page. Existing PayPal subscriber behavior was not exercised because valid subscriber credentials were unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-003</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Monthly - 2 EUR/month</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Opened /xtra; selected monthly radio option; clicked subscribe; observed plan-specific auth page.</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Monthly plan can be selected. The flow redirects to /xtra/mensual-con-anuncios and shows the selected monthly subscription with 4 EUR crossed out and 2 EUR/month.</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/3a0ac.webp; /tmp/computer-use/716c1.webp; /tmp/computer-use/8b686.webp; /tmp/computer-use/24ce9.webp</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Plan selection works before authentication. Stripe Checkout summary was not reached.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-004</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year; Annual no-ads - 30 EUR/year</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Opened /xtra; selected annual options; clicked subscribe; observed plan-specific auth pages.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Annual plans can be selected. The flow redirects to /xtra/anual-con-anuncios for 15 EUR/year and /xtra/anual-sin-anuncios for 30 EUR/year.</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/c1a65.webp; /tmp/computer-use/e219c.webp; /tmp/computer-use/105dd.webp; /tmp/computer-use/5d469.webp</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Plan selection works before authentication. Stripe Checkout summary was not reached.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-005</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Monthly and annual plans</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Inspected all plan options and compared displayed landing/auth prices.</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Displayed prices match landing/auth page expectations: monthly 4 EUR crossed out to 2 EUR/month; annual 30 EUR crossed out to 15 EUR/year; annual no-ads 60 EUR crossed out to 30 EUR/year. Discount messaging states 50 percent discount while subscription remains active.</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/d5630.webp; /tmp/computer-use/716c1.webp; /tmp/computer-use/24ce9.webp; /tmp/computer-use/5d469.webp</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Visible price mapping passed on Xataka pages. Stripe Price IDs/session summary could not be verified because checkout was not reached.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-006</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Attempted to reach checkout from subscription CTA; stopped at auth wall.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Unable to verify hosted checkout mode. All subscription attempts stayed on Xataka auth pages; checkout.stripe.com was not reached.</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp; /tmp/computer-use/a5800.webp</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Needs valid verified account to proceed past auth and inspect the payment page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-007</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Attempted QA accounts: testi.n.g.2.4.aug@gmail.com; testing24au.g2.6@gmail.com. Both rejected by login form.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Attempted login with both provided QA accounts from the subscription auth page.</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Both provided QA accounts were rejected with the message: Tu correo electronico o tu contrasena no son correctos. Logged-in Stripe Checkout email prefill could not be verified.</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/02011.webp; /tmp/computer-use/71a68.webp</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Provide a valid verified account to test email prefill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-008</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Started checkout as unauthenticated visitor; observed Xataka auth wall.</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Anonymous Stripe Checkout email field could not be observed because the flow stayed on Xataka authentication/registration before Stripe Checkout.</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Checkout email behavior requires reaching Stripe Checkout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-009</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Inspected public and auth pages; Stripe summary not reached.</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Stripe order summary with trial could not be observed. No trial messaging was visible on landing/auth pages.</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Requires checkout access and a plan configured with active trial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-010</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Attempted to proceed to checkout; stopped at auth wall.</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Stripe order summary without trial could not be observed because Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Requires checkout access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-011</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Attempted to reach checkout; stopped before Stripe domain.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Cancel/back behavior from Stripe Checkout could not be tested because Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Requires checkout access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-012</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>4000056655665556; 2223003122003222 (not used)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Attempted to reach payment submission path; stopped before Stripe Checkout.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Successful checkout and welcome redirect could not be tested because Stripe Checkout was not reached. Cards 4000056655665556 and 2223003122003222 were not entered or submitted because Stripe Checkout was not reached and test/sandbox mode was not confirmed.</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Payment submission requires verified account and confirmed Stripe test/sandbox checkout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-013</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Not executable after auth/checkout blocker.</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Account association after successful checkout could not be verified because checkout completion was not possible.</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Requires successful checkout completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-002</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:59 UTC</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-014</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>N/A - unauthenticated public flow</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Production - www.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Not executable after auth/checkout blocker.</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate activation prevention could not be tested because no checkout success URL/session was created.</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/263da.webp</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Requires completed checkout and success URL/session replay.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record testing site access blocker for Stripe retest
Co-authored-by: ShobhaAml <ShobhaAml@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
+++ b/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
@@ -603,7 +603,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RUN-STR-20261021-002</t>
+          <t>RUN-STR-20261021-003</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1. Stripe Checkout Entry and Plan Selection</t>
+          <t>1. Stripe Checkout Entry and Plan Selection via testing.xataka.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Latest blocker</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>testing.xataka.com requires HTTP Basic Auth credentials before app login.</t>
         </is>
       </c>
     </row>
@@ -1688,17 +1700,17 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Annual no-ads - 30 EUR/year</t>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -1708,22 +1720,22 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>Subscribe CTA is visible and clickable, but clicking it redirected to Xataka auth page (/xtra/anual-sin-anuncios), not checkout.stripe.com. Stripe Checkout was not reached; flow stopped at Xataka authentication wall before checkout.stripe.com.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/d5630.webp; /tmp/computer-use/263da.webp; /tmp/computer-use/a5800.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>Authentication gate prevents confirming direct Stripe Checkout redirect for visitor flow.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -1758,24 +1770,24 @@
           <t>PayPal remains available for existing subscribers; Stripe is available for new subscription checkout.</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Landing page plans</t>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -1785,22 +1797,22 @@
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Landing page shows payment text: Paga con tarjeta o PayPal, cancela cuando quieras.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/d5630.webp; /tmp/computer-use/716c1.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>PayPal coexistence is visible on the landing page. Existing PayPal subscriber behavior was not exercised because valid subscriber credentials were unavailable.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -1835,24 +1847,24 @@
           <t>Stripe Checkout order summary shows monthly plan name, monthly price and monthly billing frequency.</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Monthly - 2 EUR/month</t>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1862,22 +1874,22 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>Monthly plan can be selected. The flow redirects to /xtra/mensual-con-anuncios and shows the selected monthly subscription with 4 EUR crossed out and 2 EUR/month.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/3a0ac.webp; /tmp/computer-use/716c1.webp; /tmp/computer-use/8b686.webp; /tmp/computer-use/24ce9.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>Plan selection works before authentication. Stripe Checkout summary was not reached.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -1912,24 +1924,24 @@
           <t>Stripe Checkout order summary shows annual plan name, annual price and annual billing frequency.</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Annual with ads - 15 EUR/year; Annual no-ads - 30 EUR/year</t>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1939,22 +1951,22 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>Annual plans can be selected. The flow redirects to /xtra/anual-con-anuncios for 15 EUR/year and /xtra/anual-sin-anuncios for 30 EUR/year.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/c1a65.webp; /tmp/computer-use/e219c.webp; /tmp/computer-use/105dd.webp; /tmp/computer-use/5d469.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>Plan selection works before authentication. Stripe Checkout summary was not reached.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -1989,24 +2001,24 @@
           <t>Each plan maps to the correct Stripe Price ID and displayed amount.</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Monthly and annual plans</t>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -2016,22 +2028,22 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Displayed prices match landing/auth page expectations: monthly 4 EUR crossed out to 2 EUR/month; annual 30 EUR crossed out to 15 EUR/year; annual no-ads 60 EUR crossed out to 30 EUR/year. Discount messaging states 50 percent discount while subscription remains active.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/d5630.webp; /tmp/computer-use/716c1.webp; /tmp/computer-use/24ce9.webp; /tmp/computer-use/5d469.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>Visible price mapping passed on Xataka pages. Stripe Price IDs/session summary could not be verified because checkout was not reached.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -2073,42 +2085,42 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>Unable to verify hosted checkout mode. All subscription attempts stayed on Xataka auth pages; checkout.stripe.com was not reached.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/263da.webp; /tmp/computer-use/a5800.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>Needs valid verified account to proceed past auth and inspect the payment page.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -2150,42 +2162,42 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Attempted QA accounts: testi.n.g.2.4.aug@gmail.com; testing24au.g2.6@gmail.com. Both rejected by login form.</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Both provided QA accounts were rejected with the message: Tu correo electronico o tu contrasena no son correctos. Logged-in Stripe Checkout email prefill could not be verified.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/02011.webp; /tmp/computer-use/71a68.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>Provide a valid verified account to test email prefill.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -2227,42 +2239,42 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Anonymous Stripe Checkout email field could not be observed because the flow stayed on Xataka authentication/registration before Stripe Checkout.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/263da.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>Checkout email behavior requires reaching Stripe Checkout.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -2304,42 +2316,42 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Stripe order summary with trial could not be observed. No trial messaging was visible on landing/auth pages.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/263da.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>Requires checkout access and a plan configured with active trial.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -2381,42 +2393,42 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>Stripe order summary without trial could not be observed because Stripe Checkout was not reached.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/263da.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>Requires checkout access.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -2458,42 +2470,42 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>Cancel/back behavior from Stripe Checkout could not be tested because Stripe Checkout was not reached.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/263da.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>Requires checkout access.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -2535,17 +2547,17 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -2555,22 +2567,22 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>Successful checkout and welcome redirect could not be tested because Stripe Checkout was not reached. Cards 4000056655665556 and 2223003122003222 were not entered or submitted because Stripe Checkout was not reached and test/sandbox mode was not confirmed.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/263da.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>Payment submission requires verified account and confirmed Stripe test/sandbox checkout.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -2612,42 +2624,42 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Account association after successful checkout could not be verified because checkout completion was not possible.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/263da.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>Requires successful checkout completion.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -2689,42 +2701,42 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:59 UTC</t>
+          <t>2026-10-21 08:53 UTC</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>N/A - unauthenticated public flow</t>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra</t>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Duplicate activation prevention could not be tested because no checkout success URL/session was created.</t>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/263da.webp</t>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
-          <t>Requires completed checkout and success URL/session replay.</t>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
         </is>
       </c>
     </row>
@@ -6014,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7147,6 +7159,874 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-001</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-002</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-003</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-004</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-005</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-006</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-007</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-008</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-009</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-010</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-011</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-012</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>4000056655665556; 2223003122003222 (not used)</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-013</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-003</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:53 UTC</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-014</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>N/A - testing site inaccessible before XTRA landing page</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/; encountered HTTP Basic Auth prompt; attempted provided app account and common server credentials; all attempts failed; stopped before XTRA landing page.</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record successful Stripe sandbox payment retest
Co-authored-by: ShobhaAml <ShobhaAml@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
+++ b/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,8 +45,16 @@
       <b val="1"/>
       <color rgb="00274E13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00666666"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +74,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -127,6 +145,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -494,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -572,7 +596,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
@@ -592,7 +616,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
@@ -603,7 +627,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RUN-STR-20261021-003</t>
+          <t>RUN-STR-20261021-004</t>
         </is>
       </c>
     </row>
@@ -615,7 +639,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1. Stripe Checkout Entry and Plan Selection via testing.xataka.com</t>
+          <t>1. Stripe Checkout Entry and Plan Selection via testing.xataka.com Sandbox</t>
         </is>
       </c>
     </row>
@@ -627,8 +651,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>testing.xataka.com requires HTTP Basic Auth credentials before app login.</t>
-        </is>
+          <t>TC-STR-010 blocked because no no-trial plan was available; TC-STR-008 requires anonymous session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Not run test cases</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Partial test cases</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1578,7 +1622,7 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
-    <col width="47" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
     <col width="55" customWidth="1" min="12" max="12"/>
     <col width="55" customWidth="1" min="13" max="13"/>
     <col width="55" customWidth="1" min="14" max="14"/>
@@ -1693,24 +1737,24 @@
           <t>User is redirected to Stripe Checkout on checkout.stripe.com.</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Annual with ads - 15 EUR/year</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -1720,22 +1764,22 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Subscription CTA/payment path reached Stripe Checkout at checkout.stripe.com in Sandbox mode.</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/405f4.webp; /tmp/computer-use/98149.webp</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>HTTP Basic Auth succeeded. App login succeeded. Stripe Checkout displayed Sandbox badge; no real charges were made.</t>
         </is>
       </c>
     </row>
@@ -1770,24 +1814,24 @@
           <t>PayPal remains available for existing subscribers; Stripe is available for new subscription checkout.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Landing page plans</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -1797,22 +1841,22 @@
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Landing page/payment page showed card and PayPal coexistence text/options.</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/6e9da.webp</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>Text observed: Paga con tarjeta o PayPal, cancela cuando quieras.</t>
         </is>
       </c>
     </row>
@@ -1847,24 +1891,24 @@
           <t>Stripe Checkout order summary shows monthly plan name, monthly price and monthly billing frequency.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Monthly - 2 EUR/month</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1874,22 +1918,22 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Monthly plan selection worked via /xtra/mensual-con-anuncios. Stripe Checkout summary showed Xataka Xtra, 1 day free trial, then $2.34/month after trial.</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/4f832.webp; /tmp/computer-use/4f336.webp; /tmp/computer-use/a3b73.webp</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>Direct /xtra/mensual URL returned 404, but selecting the monthly radio option from XTRA worked correctly.</t>
         </is>
       </c>
     </row>
@@ -1924,24 +1968,24 @@
           <t>Stripe Checkout order summary shows annual plan name, annual price and annual billing frequency.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Annual with ads - 15 EUR/year; Annual no-ads - 30 EUR/year</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1951,22 +1995,22 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Annual plan selection worked for both annual variants and opened Stripe Checkout.</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/6e9da.webp; /tmp/computer-use/98149.webp; /tmp/computer-use/bb63a.webp</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>HTTP Basic Auth succeeded. App login succeeded. Stripe Checkout displayed Sandbox badge; no real charges were made.</t>
         </is>
       </c>
     </row>
@@ -2001,24 +2045,24 @@
           <t>Each plan maps to the correct Stripe Price ID and displayed amount.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Monthly and annual plans</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -2028,22 +2072,22 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Displayed plan amounts matched tested selections: monthly 2 EUR/month shown as $2.34/month after trial; annual with ads 15 EUR shown as $17.52; annual no-ads 30 EUR shown as $35.04.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/6e9da.webp; /tmp/computer-use/a3b73.webp; /tmp/computer-use/98149.webp; /tmp/computer-use/bb63a.webp</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>Stripe session displayed corresponding converted amounts. Stripe Price IDs were not exposed in the UI.</t>
         </is>
       </c>
     </row>
@@ -2078,24 +2122,24 @@
           <t>Payment UI is hosted by Stripe; Xataka does not render or collect card fields locally.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Annual with ads; Annual no-ads; Monthly</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -2105,22 +2149,22 @@
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Payment UI was hosted on Stripe Checkout at checkout.stripe.com. Card number, expiry, CVC, name, and ZIP fields were displayed by Stripe.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/98149.webp; /tmp/computer-use/bb63a.webp; /tmp/computer-use/a3b73.webp</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>No local Xataka card-entry UI was observed.</t>
         </is>
       </c>
     </row>
@@ -2155,24 +2199,24 @@
           <t>Email field is pre-filled with logged-in user email.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Annual with ads; Monthly</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -2182,22 +2226,22 @@
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Stripe Checkout email field was prefilled with the logged-in user email.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/98149.webp; /tmp/computer-use/a3b73.webp</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>HTTP Basic Auth succeeded. App login succeeded. Stripe Checkout displayed Sandbox badge; no real charges were made.</t>
         </is>
       </c>
     </row>
@@ -2232,24 +2276,24 @@
           <t>Checkout allows user to enter email or follows configured authentication flow.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -2259,22 +2303,22 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Anonymous checkout email behavior was not tested because the current run used an authenticated session.</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/a3b73.webp</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>Requires anonymous/incognito session or explicit logout before retest.</t>
         </is>
       </c>
     </row>
@@ -2309,24 +2353,24 @@
           <t>Stripe Checkout summary shows plan name, price, billing frequency and trial period.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Monthly and annual plans</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -2336,22 +2380,22 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Stripe Checkout order summaries displayed plan amount/frequency and 1 day free trial messaging.</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/a3b73.webp; /tmp/computer-use/98149.webp; /tmp/computer-use/bb63a.webp</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>All tested plans showed trial messaging.</t>
         </is>
       </c>
     </row>
@@ -2393,17 +2437,17 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>All visible plans</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -2413,22 +2457,22 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>No plan without trial messaging was available. Monthly and both annual plans all displayed 1 day free trial messaging in Stripe Checkout.</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/a3b73.webp; /tmp/computer-use/bb63a.webp</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>Cannot execute no-trial summary test until a no-trial plan/configuration is available.</t>
         </is>
       </c>
     </row>
@@ -2463,24 +2507,24 @@
           <t>User returns to Xataka subscription page.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Annual no-ads - 30 EUR/year</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -2490,22 +2534,22 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Stripe Checkout back/cancel action returned to the merchant site at testing.xataka.com/xtra/anual-sin-anuncios, and further navigation returned to XTRA landing.</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/bb63a.webp; /tmp/computer-use/a74b5.webp</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>Cancel/back did not complete payment.</t>
         </is>
       </c>
     </row>
@@ -2540,49 +2584,49 @@
           <t>User returns to Xataka success/welcome page.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Annual with ads - 15 EUR/year; Annual no-ads - 30 EUR/year</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>4000056655665556; 2223003122003222 (not used)</t>
+          <t>4000056655665556; 2223003122003222</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Successful sandbox card payments completed with both provided cards and redirected to Xataka success flow.</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/ab931.webp; /tmp/computer-use/3c1a1.webp; /tmp/computer-use/7981a.webp; /tmp/computer-use/16b57.webp</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>Stripe Sandbox badge confirmed before submission; no real charge was made.</t>
         </is>
       </c>
     </row>
@@ -2617,49 +2661,49 @@
           <t>Xataka account is associated with active Stripe subscription/customer.</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Monthly and annual flows after successful payments</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>4000056655665556; 2223003122003222</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Post-payment user profile/flow showed subscription selection for the logged-in account, and success URL redirected back to XTRA. Full backend/customer association was not directly inspectable from the UI.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/8a1ef.webp; /tmp/computer-use/d8ac6.webp</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>UI evidence suggests account association, but backend Stripe customer/subscription linkage was not independently verified.</t>
         </is>
       </c>
     </row>
@@ -2694,24 +2738,24 @@
           <t>No duplicate subscription or duplicate activation is created.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 08:53 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Application QA accounts attempted against HTTP Basic Auth: testi.n.g.2.4.aug@gmail.com. Additional common HTTP Basic Auth combinations xataka/xataka and test/test also failed. testing24au.g2.6@gmail.com was not reached at app login because server auth blocked access.</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>N/A - testing site inaccessible before XTRA landing page</t>
+          <t>Post-success URL</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -2721,22 +2765,22 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/ (blocked by HTTP Basic Authentication)</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Testing site could not be accessed. Browser displayed HTTP Basic Authentication prompt for https://testing.xataka.com and rejected attempted credentials. XTRA landing page, application login, and Stripe Checkout were not reached.</t>
+          <t>Revisiting /xtra/success redirected to XTRA landing and did not create a new checkout session, duplicate activation warning, or visible duplicate flow.</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/89cf6.webp; /tmp/computer-use/5a88b.webp; /tmp/computer-use/f1a6e.webp; /tmp/computer-use/1eaf9.webp</t>
+          <t>/tmp/computer-use/8dba2.webp; /tmp/computer-use/d8ac6.webp; /tmp/computer-use/3da15.webp</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
-          <t>Provide the correct HTTP Basic Auth username/password for testing.xataka.com, or a testing URL without server-level auth. Cards 4000056655665556 and 2223003122003222 were not entered or submitted.</t>
+          <t>UI-level duplicate activation prevention passed; backend duplicate-subscription data was not directly inspected.</t>
         </is>
       </c>
     </row>
@@ -2771,19 +2815,19 @@
           <t>Payment succeeds and subscription activates.</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:38 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Provided accounts failed: testi.n.g.2.4.aug@gmail.com; testing24au.g2.6@gmail.com. New account created: xatratest21oct@gmail.com (blocked at email verification).</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -2798,22 +2842,22 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra; payment checkout not reached</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Stripe Checkout was not reached. The subscription flow stopped before payment because both provided QA logins were rejected, and the newly created account required email verification before checkout access. Card entry/payment could not be executed.</t>
+          <t>Sandbox card payment succeeded and redirected to Xataka success flow.</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/feeb6.webp; /tmp/computer-use/8f35c.webp; /tmp/computer-use/b71c0.webp</t>
+          <t>/tmp/computer-use/ab931.webp; /tmp/computer-use/3c1a1.webp</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>Do not submit card details until a verified QA account reaches Stripe Checkout and test/sandbox mode is confirmed. Unblock by providing a verified Xataka test account or mailbox access for xatratest21oct@gmail.com.</t>
+          <t>Card entered only after Stripe Sandbox mode was confirmed.</t>
         </is>
       </c>
     </row>
@@ -2848,24 +2892,24 @@
           <t>Payment succeeds and subscription activates.</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 07:38 UTC</t>
+          <t>2026-10-21 17:47 UTC</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Provided accounts failed: testi.n.g.2.4.aug@gmail.com; testing24au.g2.6@gmail.com. New account created: xatratest21oct@gmail.com (blocked at email verification).</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Annual with ads - 15 EUR/year</t>
+          <t>Annual no-ads - 30 EUR/year</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -2875,22 +2919,22 @@
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>Production - www.xataka.com/xtra; payment checkout not reached</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
         </is>
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>Stripe Checkout was not reached. The subscription flow stopped before payment because both provided QA logins were rejected, and the newly created account required email verification before checkout access. Card entry/payment could not be executed.</t>
+          <t>Sandbox card payment succeeded and redirected to Xataka success flow.</t>
         </is>
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/feeb6.webp; /tmp/computer-use/8f35c.webp; /tmp/computer-use/b71c0.webp</t>
+          <t>/tmp/computer-use/7981a.webp; /tmp/computer-use/16b57.webp</t>
         </is>
       </c>
       <c r="O17" s="5" t="inlineStr">
         <is>
-          <t>Do not submit card details until a verified QA account reaches Stripe Checkout and test/sandbox mode is confirmed. Unblock by providing a verified Xataka test account or mailbox access for xatratest21oct@gmail.com.</t>
+          <t>Card entered only after Stripe Sandbox mode was confirmed. Card network displayed as Mastercard.</t>
         </is>
       </c>
     </row>
@@ -6026,7 +6070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8027,6 +8071,998 @@
         </is>
       </c>
     </row>
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-001</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Logged into testing site; opened XTRA; selected annual plan; clicked card payment; observed Stripe Checkout.</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>Subscription CTA/payment path reached Stripe Checkout at checkout.stripe.com in Sandbox mode.</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/405f4.webp; /tmp/computer-use/98149.webp</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>HTTP Basic Auth succeeded. App login succeeded. Stripe Checkout displayed Sandbox badge; no real charges were made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="45" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-002</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Landing page plans</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Opened XTRA landing page and inspected available payment/subscription messaging.</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Landing page/payment page showed card and PayPal coexistence text/options.</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/6e9da.webp</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>Text observed: Paga con tarjeta o PayPal, cancela cuando quieras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="45" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-003</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Monthly - 2 EUR/month</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Selected monthly radio option; clicked subscription CTA; clicked card payment; observed monthly Stripe Checkout summary.</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>Monthly plan selection worked via /xtra/mensual-con-anuncios. Stripe Checkout summary showed Xataka Xtra, 1 day free trial, then $2.34/month after trial.</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/4f832.webp; /tmp/computer-use/4f336.webp; /tmp/computer-use/a3b73.webp</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>Direct /xtra/mensual URL returned 404, but selecting the monthly radio option from XTRA worked correctly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="45" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-004</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year; Annual no-ads - 30 EUR/year</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Selected annual plan options from XTRA and proceeded to payment/Stripe Checkout.</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>Annual plan selection worked for both annual variants and opened Stripe Checkout.</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/6e9da.webp; /tmp/computer-use/98149.webp; /tmp/computer-use/bb63a.webp</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>HTTP Basic Auth succeeded. App login succeeded. Stripe Checkout displayed Sandbox badge; no real charges were made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="45" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-005</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Monthly and annual plans</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Inspected XTRA plan prices and Stripe Checkout summaries for monthly and annual variants.</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>Displayed plan amounts matched tested selections: monthly 2 EUR/month shown as $2.34/month after trial; annual with ads 15 EUR shown as $17.52; annual no-ads 30 EUR shown as $35.04.</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/6e9da.webp; /tmp/computer-use/a3b73.webp; /tmp/computer-use/98149.webp; /tmp/computer-use/bb63a.webp</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>Stripe session displayed corresponding converted amounts. Stripe Price IDs were not exposed in the UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-006</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads; Annual no-ads; Monthly</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Opened card payment flow and inspected payment domain/UI.</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>Payment UI was hosted on Stripe Checkout at checkout.stripe.com. Card number, expiry, CVC, name, and ZIP fields were displayed by Stripe.</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/98149.webp; /tmp/computer-use/bb63a.webp; /tmp/computer-use/a3b73.webp</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>No local Xataka card-entry UI was observed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-007</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads; Monthly</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Logged in with QA user; opened Stripe Checkout; inspected email field.</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Checkout email field was prefilled with the logged-in user email.</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/98149.webp; /tmp/computer-use/a3b73.webp</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>HTTP Basic Auth succeeded. App login succeeded. Stripe Checkout displayed Sandbox badge; no real charges were made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-008</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Observed authenticated checkout only; no logout/incognito anonymous test was performed.</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>Anonymous checkout email behavior was not tested because the current run used an authenticated session.</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/a3b73.webp</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>Requires anonymous/incognito session or explicit logout before retest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="45" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-009</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Monthly and annual plans</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Opened monthly and annual Stripe Checkout summaries and inspected trial/price details.</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Checkout order summaries displayed plan amount/frequency and 1 day free trial messaging.</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/a3b73.webp; /tmp/computer-use/98149.webp; /tmp/computer-use/bb63a.webp</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>All tested plans showed trial messaging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="45" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-010</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>All visible plans</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Checked monthly, annual with ads, and annual no-ads Stripe Checkout summaries.</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>No plan without trial messaging was available. Monthly and both annual plans all displayed 1 day free trial messaging in Stripe Checkout.</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/a3b73.webp; /tmp/computer-use/bb63a.webp</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>Cannot execute no-trial summary test until a no-trial plan/configuration is available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-011</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Annual no-ads - 30 EUR/year</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>Opened Stripe Checkout; clicked Stripe back arrow; observed return to merchant site.</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Checkout back/cancel action returned to the merchant site at testing.xataka.com/xtra/anual-sin-anuncios, and further navigation returned to XTRA landing.</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/bb63a.webp; /tmp/computer-use/a74b5.webp</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>Cancel/back did not complete payment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="45" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-012</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year; Annual no-ads - 30 EUR/year</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>4000056655665556; 2223003122003222</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Entered card 4000056655665556 for annual with ads; submitted; observed success. Repeated with card 2223003122003222 for annual no-ads; observed success.</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>Successful sandbox card payments completed with both provided cards and redirected to Xataka success flow.</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/ab931.webp; /tmp/computer-use/3c1a1.webp; /tmp/computer-use/7981a.webp; /tmp/computer-use/16b57.webp</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Sandbox badge confirmed before submission; no real charge was made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="45" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-013</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Monthly and annual flows after successful payments</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>4000056655665556; 2223003122003222</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>After successful payments, navigated to XTRA and /xtra/success; inspected visible logged-in state and redirect behavior.</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>Post-payment user profile/flow showed subscription selection for the logged-in account, and success URL redirected back to XTRA. Full backend/customer association was not directly inspectable from the UI.</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/8a1ef.webp; /tmp/computer-use/d8ac6.webp</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>UI evidence suggests account association, but backend Stripe customer/subscription linkage was not independently verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="45" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>TC-STR-014</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Post-success URL</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Directly opened testing.xataka.com/xtra/success after completed checkout and observed redirect/final state.</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>Revisiting /xtra/success redirected to XTRA landing and did not create a new checkout session, duplicate activation warning, or visible duplicate flow.</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/8dba2.webp; /tmp/computer-use/d8ac6.webp; /tmp/computer-use/3da15.webp</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>UI-level duplicate activation prevention passed; backend duplicate-subscription data was not directly inspected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="45" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-001</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>4000056655665556</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Opened Stripe Sandbox Checkout; entered card 4000056655665556; submitted payment; observed success redirect.</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>Sandbox card payment succeeded and redirected to Xataka success flow.</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/ab931.webp; /tmp/computer-use/3c1a1.webp</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>Card entered only after Stripe Sandbox mode was confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="45" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261021-004</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47 UTC</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-002</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Annual no-ads - 30 EUR/year</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Opened Stripe Sandbox Checkout; entered card 2223003122003222; submitted payment; observed success redirect.</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>Sandbox card payment succeeded and redirected to Xataka success flow.</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/computer-use/7981a.webp; /tmp/computer-use/16b57.webp</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>Card entered only after Stripe Sandbox mode was confirmed. Card network displayed as Mastercard.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record card payment and error execution results
Co-authored-by: ShobhaAml <ShobhaAml@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
+++ b/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +53,12 @@
       <b val="1"/>
       <color rgb="007F6000"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00990000"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +88,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -127,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -151,6 +160,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -586,7 +598,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
@@ -596,7 +608,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
@@ -606,7 +618,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
@@ -616,7 +628,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
@@ -627,7 +639,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RUN-STR-20261021-004</t>
+          <t>RUN-STR-20261022-005</t>
         </is>
       </c>
     </row>
@@ -639,7 +651,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1. Stripe Checkout Entry and Plan Selection via testing.xataka.com Sandbox</t>
+          <t>2. Card Payment Method and Payment Errors</t>
         </is>
       </c>
     </row>
@@ -651,7 +663,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TC-STR-010 blocked because no no-trial plan was available; TC-STR-008 requires anonymous session.</t>
+          <t>TC-PAY-008 needs Stripe Dashboard or test-clock access. TC-PAY-004 failed because invalid expiry 13/20 was rewritten to 01/32 without an error.</t>
         </is>
       </c>
     </row>
@@ -672,7 +684,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1613,7 +1625,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="47" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
@@ -1622,7 +1634,7 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="54" customWidth="1" min="11" max="11"/>
     <col width="55" customWidth="1" min="12" max="12"/>
     <col width="55" customWidth="1" min="13" max="13"/>
     <col width="55" customWidth="1" min="14" max="14"/>
@@ -2822,42 +2834,42 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 17:47 UTC</t>
+          <t>2026-10-22 07:18 UTC</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>testi.n.g.2.4.aug@gmail.com</t>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Annual with ads - 15 EUR/year</t>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>4000056655665556</t>
+          <t>4242424242424242</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Sandbox card payment succeeded and redirected to Xataka success flow.</t>
+          <t>Sandbox credit-card checkout completed. Stripe showed Entorno de prueba, then redirected to https://testing.xataka.com/xtra/success with a cs_test_ session id. This was the standard Stripe credit test card; the user-supplied cards are debit cards and were used for TC-PAY-002.</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/ab931.webp; /tmp/computer-use/3c1a1.webp</t>
+          <t>/tmp/section2/05-stripe-or-blocker.png; /tmp/section2/13-credit-result.png</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>Card entered only after Stripe Sandbox mode was confirmed.</t>
+          <t>Success URL: /xtra/success?session_id=cs_test_b184VAPjkmYPtr8CIq9XPdGE0q1ae2uEMWGm02PERdMaEdpcvzY1BJ9M8I. A later debit payment became the card stored on the subscription.</t>
         </is>
       </c>
     </row>
@@ -2899,42 +2911,42 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 17:47 UTC</t>
+          <t>2026-10-22 07:18 UTC</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>testi.n.g.2.4.aug@gmail.com</t>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Annual no-ads - 30 EUR/year</t>
+          <t>Annual with ads - 15 EUR/year</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>2223003122003222</t>
+          <t>4000056655665556</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox/Test mode confirmed</t>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
         </is>
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>Sandbox card payment succeeded and redirected to Xataka success flow.</t>
+          <t>Visa debit sandbox payment completed. Checkout showed the card as Visa and the button changed to Procesando. Stripe test Billing Portal then showed an active Xataka Xtra subscription at 15.00 EUR/year, payment method Visa •••• 5556 expiring 12/2034, and a paid invoice for 17.54 USD on 22 Oct 2026. Next billing date is 22 Oct 2027.</t>
         </is>
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
-          <t>/tmp/computer-use/7981a.webp; /tmp/computer-use/16b57.webp</t>
+          <t>/tmp/section2/13-debit-visa-result.png; /tmp/section2/27-payment-method.png</t>
         </is>
       </c>
       <c r="O17" s="5" t="inlineStr">
         <is>
-          <t>Card entered only after Stripe Sandbox mode was confirmed. Card network displayed as Mastercard.</t>
+          <t>2223003122003222 was not reused in this run. The supplied Visa debit card completed and is the active payment method.</t>
         </is>
       </c>
     </row>
@@ -2969,6 +2981,51 @@
           <t>Stripe shows real-time validation error.</t>
         </is>
       </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>4242 (incomplete)</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Checkout showed the real-time Spanish validation message: El número de tarjeta está incompleto. Payment was not submitted.</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/06-card-number-validation.png</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Validated on hosted Stripe Checkout in test mode.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -3001,6 +3058,51 @@
           <t>Stripe shows real-time validation error.</t>
         </is>
       </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>4242424242424242</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Entering invalid expiry 13/20 did not produce a real-time validation error. Stripe normalized the entry and displayed 01/32. A follow-up with an explicitly expired date could not be repeated: both QA accounts then had active subscriptions, and Cambiar de plan returned Ha ocurrido un error y no se ha podido cambiar el plan.</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/07-expiry-validation.png; /tmp/section2/33-after-plan-action.png</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Expected a real-time invalid or expired expiry error. The invalid month was rewritten instead of rejected.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -3033,6 +3135,51 @@
           <t>Stripe shows real-time validation error.</t>
         </is>
       </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>4242424242424242</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Checkout showed the real-time Spanish validation message: El código de seguridad de la tarjeta está incompleto. Payment was not submitted.</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/08-cvc-validation.png</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Validated on hosted Stripe Checkout in test mode.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -3065,6 +3212,51 @@
           <t>User sees payment error message in user's language.</t>
         </is>
       </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>4000000000000002</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Checkout rejected the sandbox decline card with a Spanish message: Se ha rechazado tu tarjeta de crédito. Intenta pagar con una tarjeta de débito.</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/10-decline-result.png</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>Message is in the checkout language. The decline did not redirect to the Xataka success page.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -3097,6 +3289,51 @@
           <t>Subscription is not activated and premium content remains blocked.</t>
         </is>
       </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads checkout, not activated by the decline</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>4000000000000002</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Immediately after the declined checkout, the subscription page showed the public plan-selection landing and no active subscription. The failed payment did not activate Xtra. A separate later successful payment did activate the account.</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/11-after-decline-account.png</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>Premium article access was not opened separately. The account state after the decline had no active plan.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -3129,6 +3366,51 @@
           <t>Stripe retry behavior applies according to Stripe Billing configuration.</t>
         </is>
       </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Billing renewal retry could not be triggered. The storefront exposes Checkout and the test billing portal, but not Stripe test clocks, invoice retry controls, or Smart Retry configuration.</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/27-payment-method.png</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>A checkout decline is not the renewal-retry scenario. Needs Stripe Dashboard or test-clock access.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -3159,6 +3441,51 @@
       <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Xataka does not receive or store raw card data.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>4242424242424242; 4000000000000002; 4000056655665556</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>Card number, expiry, and CVC were entered only on checkout.stripe.com. Browser requests to testing.xataka.com did not contain those raw card numbers. Xataka server logs and database were not inspected.</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/05-stripe-or-blocker.png; /tmp/section2/10-decline-result.png</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>Hosted Checkout was confirmed. This does not include a server-side log or database inspection.</t>
         </is>
       </c>
     </row>
@@ -6070,16 +6397,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="47" customWidth="1" min="7" max="7"/>
+    <col width="54" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
@@ -9063,6 +9390,564 @@
         </is>
       </c>
     </row>
+    <row r="49" ht="45" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-005</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-001</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>4242424242424242</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Logged in on testing.xataka.com, selected annual with ads, opened Stripe Checkout, confirmed test mode, submitted 4242424242424242 with expiry 12/34 and CVC 123.</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>Sandbox credit-card checkout completed. Stripe showed Entorno de prueba, then redirected to https://testing.xataka.com/xtra/success with a cs_test_ session id. This was the standard Stripe credit test card; the user-supplied cards are debit cards and were used for TC-PAY-002.</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/05-stripe-or-blocker.png; /tmp/section2/13-credit-result.png</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>Success URL: /xtra/success?session_id=cs_test_b184VAPjkmYPtr8CIq9XPdGE0q1ae2uEMWGm02PERdMaEdpcvzY1BJ9M8I. A later debit payment became the card stored on the subscription.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="45" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-005</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-002</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>4000056655665556</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Opened a second Stripe Sandbox checkout and submitted 4000056655665556. Confirmed the resulting subscription and invoice in the Stripe test billing portal.</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>Visa debit sandbox payment completed. Checkout showed the card as Visa and the button changed to Procesando. Stripe test Billing Portal then showed an active Xataka Xtra subscription at 15.00 EUR/year, payment method Visa •••• 5556 expiring 12/2034, and a paid invoice for 17.54 USD on 22 Oct 2026. Next billing date is 22 Oct 2027.</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/13-debit-visa-result.png; /tmp/section2/27-payment-method.png</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>2223003122003222 was not reused in this run. The supplied Visa debit card completed and is the active payment method.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="45" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-005</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-003</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>4242 (incomplete)</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>Entered incomplete card number 4242 and left the field.</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Checkout showed the real-time Spanish validation message: El número de tarjeta está incompleto. Payment was not submitted.</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/06-card-number-validation.png</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>Validated on hosted Stripe Checkout in test mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="45" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-005</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-004</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>4242424242424242</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>On Stripe Checkout, entered a complete test card number and expiry 13/20, then left the field.</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>Entering invalid expiry 13/20 did not produce a real-time validation error. Stripe normalized the entry and displayed 01/32. A follow-up with an explicitly expired date could not be repeated: both QA accounts then had active subscriptions, and Cambiar de plan returned Ha ocurrido un error y no se ha podido cambiar el plan.</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/07-expiry-validation.png; /tmp/section2/33-after-plan-action.png</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>Expected a real-time invalid or expired expiry error. The invalid month was rewritten instead of rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="45" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-005</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-005</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>4242424242424242</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Entered expiry 12/34 and a one-digit CVC, then left the field.</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Checkout showed the real-time Spanish validation message: El código de seguridad de la tarjeta está incompleto. Payment was not submitted.</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/08-cvc-validation.png</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>Validated on hosted Stripe Checkout in test mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="45" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-005</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-006</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>4000000000000002</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Submitted Stripe decline test card 4000000000000002 with expiry 12/34 and CVC 123 on the confirmed test checkout.</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Checkout rejected the sandbox decline card with a Spanish message: Se ha rechazado tu tarjeta de crédito. Intenta pagar con una tarjeta de débito.</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/10-decline-result.png</t>
+        </is>
+      </c>
+      <c r="L54" s="5" t="inlineStr">
+        <is>
+          <t>Message is in the checkout language. The decline did not redirect to the Xataka success page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="45" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-005</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-007</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads checkout, not activated by the decline</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>4000000000000002</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>After the decline error remained on Stripe Checkout, opened the Xataka subscription page and checked whether a subscription had been activated.</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>Immediately after the declined checkout, the subscription page showed the public plan-selection landing and no active subscription. The failed payment did not activate Xtra. A separate later successful payment did activate the account.</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/11-after-decline-account.png</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>Premium article access was not opened separately. The account state after the decline had no active plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="45" customHeight="1">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-005</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-008</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Checked Checkout and the Stripe test billing portal for a renewal-failure or retry control.</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>Stripe Billing renewal retry could not be triggered. The storefront exposes Checkout and the test billing portal, but not Stripe test clocks, invoice retry controls, or Smart Retry configuration.</t>
+        </is>
+      </c>
+      <c r="K56" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/27-payment-method.png</t>
+        </is>
+      </c>
+      <c r="L56" s="5" t="inlineStr">
+        <is>
+          <t>A checkout decline is not the renewal-retry scenario. Needs Stripe Dashboard or test-clock access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="45" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-005</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18 UTC</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>TC-PAY-009</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year (Stripe summary 17.54 USD/year, 1 day trial on the first checkout)</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>4242424242424242; 4000000000000002; 4000056655665556</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe Checkout Sandbox confirmed (Entorno de prueba, cs_test_ session)</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>Monitored browser request bodies for the test card numbers while entering and submitting them on Stripe Checkout.</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>Card number, expiry, and CVC were entered only on checkout.stripe.com. Browser requests to testing.xataka.com did not contain those raw card numbers. Xataka server logs and database were not inspected.</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/05-stripe-or-blocker.png; /tmp/section2/10-decline-result.png</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>Hosted Checkout was confirmed. This does not include a server-side log or database inspection.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record rejected QA account login attempts
Co-authored-by: ShobhaAml <ShobhaAml@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
+++ b/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Test Cases" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Regression Checklist" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Execution Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="QA Accounts" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Use Cases'!$A$1:$D$41</definedName>
@@ -530,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -549,7 +550,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Source Markdown</t>
@@ -561,7 +562,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1">
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Use cases</t>
@@ -571,7 +572,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Test cases</t>
@@ -581,7 +582,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Regression checklist items</t>
@@ -591,7 +592,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>Executed test cases</t>
@@ -601,7 +602,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>Passed test cases</t>
@@ -611,7 +612,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>Failed test cases</t>
@@ -621,7 +622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1">
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>Blocked test cases</t>
@@ -631,7 +632,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" ht="45" customHeight="1">
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>Latest execution run</t>
@@ -639,11 +640,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RUN-STR-20261022-005</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>Latest executed section</t>
@@ -651,11 +652,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2. Card Payment Method and Payment Errors</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
+          <t>QA account login check for fresh Stripe Checkout</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>Latest blocker</t>
@@ -663,11 +664,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TC-PAY-008 needs Stripe Dashboard or test-clock access. TC-PAY-004 failed because invalid expiry 13/20 was rewritten to 01/32 without an error.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
+          <t>All 10 newly supplied accounts were rejected by the testing.xataka.com login form. TC-PAY-004 remains Fail; expiry could not be retested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>Not run test cases</t>
@@ -677,7 +678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
+    <row r="14" ht="36" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>Partial test cases</t>
@@ -685,6 +686,26 @@
       </c>
       <c r="B14" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>New QA accounts checked</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>New QA accounts accepted</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6397,12 +6418,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
@@ -6476,7 +6497,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-001</t>
@@ -6538,7 +6559,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1">
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-001</t>
@@ -6600,7 +6621,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-001</t>
@@ -6662,7 +6683,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -6724,7 +6745,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -6786,7 +6807,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -6848,7 +6869,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -6910,7 +6931,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1">
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -6972,7 +6993,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="45" customHeight="1">
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -7034,7 +7055,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1">
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -7096,7 +7117,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="45" customHeight="1">
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -7158,7 +7179,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1">
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -7220,7 +7241,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
+    <row r="14" ht="36" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -7282,7 +7303,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
+    <row r="15" ht="36" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -7344,7 +7365,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -7406,7 +7427,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="45" customHeight="1">
+    <row r="17" ht="36" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -7468,7 +7489,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="45" customHeight="1">
+    <row r="18" ht="36" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-002</t>
@@ -7530,7 +7551,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="45" customHeight="1">
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -7592,7 +7613,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="45" customHeight="1">
+    <row r="20" ht="36" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -7654,7 +7675,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="45" customHeight="1">
+    <row r="21" ht="36" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -7716,7 +7737,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="45" customHeight="1">
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -7778,7 +7799,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="45" customHeight="1">
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -7840,7 +7861,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="45" customHeight="1">
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -7902,7 +7923,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="45" customHeight="1">
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -7964,7 +7985,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="45" customHeight="1">
+    <row r="26" ht="36" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -8026,7 +8047,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="45" customHeight="1">
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -8088,7 +8109,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="45" customHeight="1">
+    <row r="28" ht="36" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -8150,7 +8171,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="45" customHeight="1">
+    <row r="29" ht="36" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -8212,7 +8233,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="45" customHeight="1">
+    <row r="30" ht="36" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -8274,7 +8295,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="45" customHeight="1">
+    <row r="31" ht="36" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -8336,7 +8357,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="45" customHeight="1">
+    <row r="32" ht="36" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-003</t>
@@ -8398,7 +8419,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="45" customHeight="1">
+    <row r="33" ht="36" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -8460,7 +8481,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="45" customHeight="1">
+    <row r="34" ht="36" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -8522,7 +8543,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="45" customHeight="1">
+    <row r="35" ht="36" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -8584,7 +8605,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="45" customHeight="1">
+    <row r="36" ht="36" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -8646,7 +8667,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="45" customHeight="1">
+    <row r="37" ht="36" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -8708,7 +8729,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="45" customHeight="1">
+    <row r="38" ht="36" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -8770,7 +8791,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="45" customHeight="1">
+    <row r="39" ht="36" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -8832,7 +8853,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="45" customHeight="1">
+    <row r="40" ht="36" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -8894,7 +8915,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="45" customHeight="1">
+    <row r="41" ht="36" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -8956,7 +8977,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="45" customHeight="1">
+    <row r="42" ht="36" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -9018,7 +9039,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="45" customHeight="1">
+    <row r="43" ht="36" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -9080,7 +9101,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="45" customHeight="1">
+    <row r="44" ht="36" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -9142,7 +9163,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="45" customHeight="1">
+    <row r="45" ht="36" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -9204,7 +9225,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="45" customHeight="1">
+    <row r="46" ht="36" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -9266,7 +9287,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="45" customHeight="1">
+    <row r="47" ht="36" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -9328,7 +9349,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="45" customHeight="1">
+    <row r="48" ht="36" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261021-004</t>
@@ -9390,7 +9411,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="45" customHeight="1">
+    <row r="49" ht="36" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261022-005</t>
@@ -9452,7 +9473,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="45" customHeight="1">
+    <row r="50" ht="36" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261022-005</t>
@@ -9514,7 +9535,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="45" customHeight="1">
+    <row r="51" ht="36" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261022-005</t>
@@ -9576,7 +9597,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="45" customHeight="1">
+    <row r="52" ht="36" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261022-005</t>
@@ -9638,7 +9659,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="45" customHeight="1">
+    <row r="53" ht="36" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261022-005</t>
@@ -9700,7 +9721,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="45" customHeight="1">
+    <row r="54" ht="36" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261022-005</t>
@@ -9762,7 +9783,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="45" customHeight="1">
+    <row r="55" ht="36" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261022-005</t>
@@ -9824,7 +9845,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="45" customHeight="1">
+    <row r="56" ht="36" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261022-005</t>
@@ -9886,7 +9907,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="45" customHeight="1">
+    <row r="57" ht="36" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
           <t>RUN-STR-20261022-005</t>
@@ -9945,6 +9966,1056 @@
       <c r="L57" s="5" t="inlineStr">
         <is>
           <t>Hosted Checkout was confirmed. This does not include a server-side log or database inspection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="36" customHeight="1">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.a.u.g.2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K58" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L58" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="36" customHeight="1">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.aug2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="36" customHeight="1">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.aug.26@gmail.com</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K60" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L60" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="36" customHeight="1">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.aug.2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="36" customHeight="1">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g26@gmail.com</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K62" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L62" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="36" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D63" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K63" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L63" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="36" customHeight="1">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g.26@gmail.com</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K64" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="36" customHeight="1">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g.2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K65" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L65" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="36" customHeight="1">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.a.ug26@gmail.com</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="36" customHeight="1">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-006</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>QA account login</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.a.ug2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Annual with ads - 15 EUR/year</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>Opened the annual-with-ads subscription page and submitted the account on the Xataka login form.</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. Stripe Checkout was not reached.</t>
+        </is>
+      </c>
+      <c r="K67" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/61-aug26.png</t>
+        </is>
+      </c>
+      <c r="L67" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Checked (UTC)</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Login result</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Message shown</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Checkout reached</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.a.u.g.2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.aug2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.aug.26@gmail.com</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.aug.2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g26@gmail.com</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g.26@gmail.com</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g.2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.a.ug26@gmail.com</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.a.ug2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:45 UTC</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record homepage login path before XTRA
Co-authored-by: ShobhaAml <ShobhaAml@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
+++ b/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
@@ -640,7 +640,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RUN-STR-20261022-006</t>
+          <t>RUN-STR-20261022-007</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>QA account login check for fresh Stripe Checkout</t>
+          <t>Homepage login at testing.xataka.com, then XTRA landing</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>All 10 newly supplied accounts were rejected by the testing.xataka.com login form. TC-PAY-004 remains Fail; expiry could not be retested.</t>
+          <t>10 newly supplied accounts are rejected on the homepage login. The known account testi.n.g.2.4.aug@gmail.com logs in and reaches XTRA with an existing annual no-ads plan.</t>
         </is>
       </c>
     </row>
@@ -6418,16 +6418,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="54" customWidth="1" min="7" max="7"/>
+    <col width="47" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
@@ -10586,6 +10586,688 @@
       <c r="L67" s="5" t="inlineStr">
         <is>
           <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Annual no-ads - existing subscription</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/, logged in from the homepage panel, then opened https://testing.xataka.com/xtra.</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>Login succeeded as deactiveaccount. XTRA landing showed Xtra: Plan anual sin anuncios. Stripe Checkout was not started.</t>
+        </is>
+      </c>
+      <c r="K68" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png; /tmp/section2/77-known-xtra-from-home.png</t>
+        </is>
+      </c>
+      <c r="L68" s="5" t="inlineStr">
+        <is>
+          <t>This confirms the required login path. The account already has an active plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.a.u.g.2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L69" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.aug2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L70" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.aug.26@gmail.com</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K71" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L71" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.aug.2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L72" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g26@gmail.com</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K73" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g.26@gmail.com</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K75" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L75" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.au.g.2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K76" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L76" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.a.ug26@gmail.com</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K77" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L77" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login then XTRA</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>testing.2.4.a.ug2.6@gmail.com</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Not reached</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>Opened https://testing.xataka.com/ and submitted the account in the homepage login panel.</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos. XTRA landing was not opened.</t>
+        </is>
+      </c>
+      <c r="K78" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/section2/75-known-after-login.png</t>
+        </is>
+      </c>
+      <c r="L78" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>
@@ -10600,7 +11282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -10608,7 +11290,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -10652,54 +11334,54 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>testing.2.4.a.u.g.2.6@gmail.com</t>
+          <t>testi.n.g.2.4.aug@gmail.com</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 07:45 UTC</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
-        <is>
-          <t>Rejected</t>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+          <t>Homepage login succeeded. Username deactiveaccount. XTRA landing shows an existing annual no-ads plan.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - existing subscription, Checkout not started</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+          <t>Logged in from the testing homepage, then opened the XTRA landing page.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>testing.2.4.aug2.6@gmail.com</t>
+          <t>testing.2.4.a.u.g.2.6@gmail.com</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 07:45 UTC</t>
+          <t>2026-10-22 08:04 UTC</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -10719,24 +11401,24 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>testing.2.4.aug.26@gmail.com</t>
+          <t>testing.2.4.aug2.6@gmail.com</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 07:45 UTC</t>
+          <t>2026-10-22 08:04 UTC</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -10756,24 +11438,24 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>testing.2.4.aug.2.6@gmail.com</t>
+          <t>testing.2.4.aug.26@gmail.com</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 07:45 UTC</t>
+          <t>2026-10-22 08:04 UTC</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -10793,24 +11475,24 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>testing.2.4.au.g26@gmail.com</t>
+          <t>testing.2.4.aug.2.6@gmail.com</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 07:45 UTC</t>
+          <t>2026-10-22 08:04 UTC</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -10830,24 +11512,24 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>testing.2.4.au.g2.6@gmail.com</t>
+          <t>testing.2.4.au.g26@gmail.com</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 07:45 UTC</t>
+          <t>2026-10-22 08:04 UTC</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -10867,24 +11549,24 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>testing.2.4.au.g.26@gmail.com</t>
+          <t>testing.2.4.au.g2.6@gmail.com</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 07:45 UTC</t>
+          <t>2026-10-22 08:04 UTC</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -10904,24 +11586,24 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>testing.2.4.au.g.2.6@gmail.com</t>
+          <t>testing.2.4.au.g.26@gmail.com</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 07:45 UTC</t>
+          <t>2026-10-22 08:04 UTC</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -10941,24 +11623,24 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>testing.2.4.a.ug26@gmail.com</t>
+          <t>testing.2.4.au.g.2.6@gmail.com</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 07:45 UTC</t>
+          <t>2026-10-22 08:04 UTC</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -10978,44 +11660,81 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>testing.2.4.a.ug26@gmail.com</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Tu correo electrónico o tu contraseña no son correctos.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
           <t>testing.2.4.a.ug2.6@gmail.com</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Testing - https://testing.xataka.com/xtra/anual-con-anuncios</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-22 07:45 UTC</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Login at https://testing.xataka.com/, then open https://testing.xataka.com/xtra</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:04 UTC</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Tu correo electrónico o tu contraseña no son correctos.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Shared password was used for the attempt and is not stored in this workbook. Stripe Checkout was not opened.</t>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record free trial and subscription lifecycle results
Co-authored-by: ShobhaAml <ShobhaAml@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
+++ b/Aml_automation/XATAKA_XTRA_STRIPE_BILLING_USE_CASES_AND_TEST_CASES.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +57,28 @@
     <font>
       <b val="1"/>
       <color rgb="00990000"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C5700"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00274E13"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="8">
@@ -137,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -164,6 +186,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -598,8 +635,8 @@
           <t>Executed test cases</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>24</v>
+      <c r="B6" s="10" t="n">
+        <v>49</v>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
@@ -608,8 +645,8 @@
           <t>Passed test cases</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>17</v>
+      <c r="B7" s="10" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
@@ -618,7 +655,7 @@
           <t>Failed test cases</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -628,8 +665,8 @@
           <t>Blocked test cases</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>3</v>
+      <c r="B9" s="10" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
@@ -638,9 +675,9 @@
           <t>Latest execution run</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>RUN-STR-20261022-007</t>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
         </is>
       </c>
     </row>
@@ -650,9 +687,9 @@
           <t>Latest executed section</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Homepage login at testing.xataka.com, then XTRA landing</t>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>3. Free Trials and 5. Subscription Lifecycle and Premium Access</t>
         </is>
       </c>
     </row>
@@ -662,9 +699,9 @@
           <t>Latest blocker</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>10 newly supplied accounts are rejected on the homepage login. The known account testi.n.g.2.4.aug@gmail.com logs in and reaches XTRA with an existing annual no-ads plan.</t>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Testing offers a 1-day trial only, so 7/14/30-day trials are blocked. No Stripe test clock for conversion, renewal, or access after the cancellation end instant. No second login for duplicate-trial checks, and no PayPal subscriber. Xataka shows canceluser as cancelled on 22 Oct 2026 while Stripe still has that plan active with the next invoice on 22 Oct 2027.</t>
         </is>
       </c>
     </row>
@@ -674,7 +711,7 @@
           <t>Not run test cases</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -684,8 +721,8 @@
           <t>Partial test cases</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>2</v>
+      <c r="B14" s="10" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1">
@@ -3510,7 +3547,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="45" customHeight="1">
+    <row r="25" ht="72" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3541,8 +3578,53 @@
           <t>Checkout and subscription details reflect 7-day trial.</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="45" customHeight="1">
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>No 7-day plan. Catalog trial is 1 day.</t>
+        </is>
+      </c>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M25" s="12" t="inlineStr">
+        <is>
+          <t>Checkout does not show a 7-day trial. Monthly Checkout showed 1 día gratis, then 2.34 USD per month. Both annual plans also showed a 1-day trial. A 7-day trial is not configured on testing.xataka.com.</t>
+        </is>
+      </c>
+      <c r="N25" s="12" t="inlineStr">
+        <is>
+          <t>TC-STR-003, TC-STR-009, TC-STR-010; /tmp/section2/05-stripe-or-blocker.png</t>
+        </is>
+      </c>
+      <c r="O25" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: configure a 7-day trial on a plan and repeat Checkout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="72" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3573,8 +3655,53 @@
           <t>Checkout and subscription details reflect 14-day trial.</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="45" customHeight="1">
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>No 14-day plan. Catalog trial is 1 day.</t>
+        </is>
+      </c>
+      <c r="K26" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L26" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M26" s="12" t="inlineStr">
+        <is>
+          <t>Checkout and subscription details do not show a 14-day trial. The testing catalog shows a 1-day trial on the monthly plan and on both annual plans.</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>TC-STR-009, TC-STR-010; /tmp/section2/05-stripe-or-blocker.png</t>
+        </is>
+      </c>
+      <c r="O26" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: configure a 14-day trial on a plan and repeat Checkout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="72" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3605,8 +3732,53 @@
           <t>Checkout and subscription details reflect 30-day trial.</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="45" customHeight="1">
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>No 30-day plan. Catalog trial is 1 day.</t>
+        </is>
+      </c>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M27" s="12" t="inlineStr">
+        <is>
+          <t>Checkout and subscription details do not show a 30-day trial. The testing catalog shows a 1-day trial on the monthly plan and on both annual plans.</t>
+        </is>
+      </c>
+      <c r="N27" s="12" t="inlineStr">
+        <is>
+          <t>TC-STR-009, TC-STR-010; /tmp/section2/05-stripe-or-blocker.png</t>
+        </is>
+      </c>
+      <c r="O27" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: configure a 30-day trial on a plan and repeat Checkout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="72" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3637,8 +3809,53 @@
           <t>Each plan uses its own configured trial duration.</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="45" customHeight="1">
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>Monthly 2 EUR; annual with ads 15 EUR; annual no ads 30 EUR. All showed 1 day.</t>
+        </is>
+      </c>
+      <c r="K28" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L28" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M28" s="12" t="inlineStr">
+        <is>
+          <t>Monthly and both annual plans showed the same 1-day trial in Stripe Checkout. Distinct per-plan trial durations are not configured, so each plan using its own duration could not be compared.</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>TC-STR-010; /tmp/section2/05-stripe-or-blocker.png</t>
+        </is>
+      </c>
+      <c r="O28" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: set different trial lengths on monthly and annual prices, then start Checkout for each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="72" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3669,8 +3886,53 @@
           <t>User has full Xtra access immediately.</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="45" customHeight="1">
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, 1-day trial</t>
+        </is>
+      </c>
+      <c r="K29" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222 (already on the trial; not re-entered)</t>
+        </is>
+      </c>
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M29" s="12" t="inlineStr">
+        <is>
+          <t>deactiveaccount opened /xtra/gestionar-suscripcion during the trial and saw Tus beneficios Xtra, including Discord, consultorio, sorteos, and newsletters. On an article, the header CTA class was xtra-cta-hd-lead js-xtra-cta and did not include is-visible.</t>
+        </is>
+      </c>
+      <c r="N29" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/01-deactive-manage.png; /tmp/section35/05-in-article.png; /tmp/section35/06-in-sorteo.png; /tmp/section35/07-in-xtra.png</t>
+        </is>
+      </c>
+      <c r="O29" s="12" t="inlineStr">
+        <is>
+          <t>Article bodies are readable without a subscription. Immediate Xtra access shows up as the subscriber area and the hidden header CTA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="72" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3701,8 +3963,53 @@
           <t>No charge is generated until trial ends.</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="45" customHeight="1">
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, 1-day trial</t>
+        </is>
+      </c>
+      <c r="K30" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="L30" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M30" s="12" t="inlineStr">
+        <is>
+          <t>The only Stripe invoice during the trial is 21 Oct 2026, 0.00 EUR, Paid, description Trial period for Xataka Xtra. No charge was generated. The portal lists Mastercard •••• 3222.</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/02-portal-deactive.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="O30" s="12" t="inlineStr">
+        <is>
+          <t>Portal was in test mode. Cancellation later did not add an invoice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="72" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3733,8 +4040,53 @@
           <t>Next renewal date is the exact trial end date.</t>
         </is>
       </c>
-    </row>
-    <row r="32" ht="45" customHeight="1">
+      <c r="G31" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, 1-day trial</t>
+        </is>
+      </c>
+      <c r="K31" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="L31" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M31" s="12" t="inlineStr">
+        <is>
+          <t>Before cancellation, the Xataka subscription page said the plan would renew on 22 Oct 2026 for 30 EUR/year. Stripe said the free trial ends Oct 22. After cancellation, Stripe says the service will no longer be available after the free trial ends on October 22, 2026. The date matches the trial end.</t>
+        </is>
+      </c>
+      <c r="N31" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/01-deactive-manage.png; /tmp/section35/02-portal-deactive.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="O31" s="12" t="inlineStr">
+        <is>
+          <t>The renewal date observed before cancellation was the trial end date, not a later billing anniversary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="72" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3765,8 +4117,53 @@
           <t>Subscription converts automatically to paid billing cycle.</t>
         </is>
       </c>
-    </row>
-    <row r="33" ht="45" customHeight="1">
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I32" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>deactiveaccount trial cancelled before the end; canceluser is already a paid annual plan</t>
+        </is>
+      </c>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M32" s="12" t="inlineStr">
+        <is>
+          <t>Automatic conversion at trial end was not observed. The deactiveaccount trial was cancelled before the end. canceluser's 22 Oct 2026 invoice for 17.54 USD was an immediate charge with no trial, not a trial conversion. No Stripe test clock is available.</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/12-portal-after-cancel.png; /tmp/section35/24-canceluser-portal-now.png</t>
+        </is>
+      </c>
+      <c r="O32" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: leave a trial uncancelled and advance a Stripe test clock to the trial end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="72" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3797,8 +4194,53 @@
           <t>Subscription does not convert to paid after trial end.</t>
         </is>
       </c>
-    </row>
-    <row r="34" ht="45" customHeight="1">
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, 1-day trial</t>
+        </is>
+      </c>
+      <c r="K33" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="L33" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M33" s="12" t="inlineStr">
+        <is>
+          <t>Cancelled the trial from /xtra/gestionar-suscripcion/cancelar-suscripcion after choosing Otra razón. Confirmation said Suscripción cancelada con éxito, and that Xtra continues until 22 Oct 2026 and will not renew. Stripe test portal shows Cancels Oct 22, 30.00 EUR per year, and says the service will no longer be available after the free trial ends. Invoice history is still only the 0.00 EUR trial invoice.</t>
+        </is>
+      </c>
+      <c r="N33" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/09-cancel-dialog.png; /tmp/section35/10-cancelled.png; /tmp/section35/11-after-cancel-manage.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="O33" s="12" t="inlineStr">
+        <is>
+          <t>Cancellation is at the end of the trial period. Volver a activar tu suscripción was not used. The post-end instant is covered by TC-LIF-007.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="72" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3829,8 +4271,53 @@
           <t>Free trial is not granted again.</t>
         </is>
       </c>
-    </row>
-    <row r="35" ht="45" customHeight="1">
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H34" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I34" s="12" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser); follow-up on testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>Annual with ads, 15 EUR/year, on the second checkout</t>
+        </is>
+      </c>
+      <c r="K34" s="12" t="inlineStr">
+        <is>
+          <t>4000056655665556 (card already stored on the paid subscription)</t>
+        </is>
+      </c>
+      <c r="L34" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M34" s="12" t="inlineStr">
+        <is>
+          <t>A later Stripe Checkout for canceluser, after a trial had already been used, showed Suscribirse a Xataka Xtra, Total a pagar hoy 17.54 USD, and no 1 día gratis line. The paid invoice is 22 Oct 2026 for 17.54 USD / 15.00 EUR. In this run, Suscríbete ahora for deactiveaccount returned to /xtra/gestionar-suscripcion while the cancelled trial is still open, and did not open another trial checkout. No payment was submitted in this run.</t>
+        </is>
+      </c>
+      <c r="N34" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section2/results.json (second checkout text); /tmp/section35/02-portal-canceluser.png; /tmp/section35/17-after-subscribe-click.png; /tmp/section35/24-canceluser-portal-now.png</t>
+        </is>
+      </c>
+      <c r="O34" s="12" t="inlineStr">
+        <is>
+          <t>The no-second-trial proof is the earlier sandbox checkout that charged immediately. This run did not submit a card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="72" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3861,8 +4348,53 @@
           <t>User remains ineligible for another free trial.</t>
         </is>
       </c>
-    </row>
-    <row r="36" ht="45" customHeight="1">
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>Not changed</t>
+        </is>
+      </c>
+      <c r="K35" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L35" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M35" s="12" t="inlineStr">
+        <is>
+          <t>Account deactivation and reactivation were not performed. The account menu shows Dar de baja, and that control was not used. The 10 newly supplied emails cannot log in, so there is no reactivated account to test.</t>
+        </is>
+      </c>
+      <c r="N35" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/13-post-home-login.png</t>
+        </is>
+      </c>
+      <c r="O35" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: deactivate and reactivate an account that already redeemed a trial, then start Checkout again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="72" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3893,8 +4425,53 @@
           <t>Duplication is detected after Stripe processing; subscription is canceled.</t>
         </is>
       </c>
-    </row>
-    <row r="37" ht="45" customHeight="1">
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>No second fresh account. 10 supplied emails are rejected at login.</t>
+        </is>
+      </c>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L36" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M36" s="12" t="inlineStr">
+        <is>
+          <t>A duplicate trial with the same card fingerprint from another account was not executed. The 10 supplied emails cannot log in, and a new trial was not submitted from the two working accounts.</t>
+        </is>
+      </c>
+      <c r="N36" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="O36" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: provide an account that can log in, then repeat Checkout in test mode with a card that already redeemed a trial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="72" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3925,8 +4502,53 @@
           <t>Refund is issued if a charge was generated.</t>
         </is>
       </c>
-    </row>
-    <row r="38" ht="45" customHeight="1">
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>Depends on TC-TRL-012</t>
+        </is>
+      </c>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M37" s="12" t="inlineStr">
+        <is>
+          <t>No duplicate-trial charge was created, so a refund could not be observed.</t>
+        </is>
+      </c>
+      <c r="N37" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="O37" s="12" t="inlineStr">
+        <is>
+          <t>Unblock with TC-TRL-012. Inspect the Stripe refund only after a duplicate charge exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="72" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3957,8 +4579,53 @@
           <t>Welcome page is not shown; frontend displays error that payment method was already used for a free trial and prompts contacting support.</t>
         </is>
       </c>
-    </row>
-    <row r="39" ht="45" customHeight="1">
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>Depends on TC-TRL-012</t>
+        </is>
+      </c>
+      <c r="J38" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K38" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L38" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M38" s="12" t="inlineStr">
+        <is>
+          <t>The post-Checkout error page for a card already used on a free trial was not reached.</t>
+        </is>
+      </c>
+      <c r="N38" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="O38" s="12" t="inlineStr">
+        <is>
+          <t>Unblock with TC-TRL-012, then read the return page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="72" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -3989,8 +4656,53 @@
           <t>Subscription is not activated.</t>
         </is>
       </c>
-    </row>
-    <row r="40" ht="45" customHeight="1">
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>Depends on TC-TRL-012</t>
+        </is>
+      </c>
+      <c r="J39" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K39" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L39" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M39" s="12" t="inlineStr">
+        <is>
+          <t>Subscription activation after duplicate-trial detection was not observed because the duplicate path was not started.</t>
+        </is>
+      </c>
+      <c r="N39" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="O39" s="12" t="inlineStr">
+        <is>
+          <t>Unblock with TC-TRL-012, then confirm the new account has no active subscription.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="72" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>3. Free Trials</t>
@@ -4019,6 +4731,51 @@
       <c r="F40" s="2" t="inlineStr">
         <is>
           <t>No welcome screens or welcome emails are sent.</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H40" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>Depends on TC-TRL-012</t>
+        </is>
+      </c>
+      <c r="J40" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K40" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L40" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M40" s="12" t="inlineStr">
+        <is>
+          <t>Welcome screens and welcome email for a duplicate trial were not observed. The duplicate path was not started, and the mailbox was not inspected.</t>
+        </is>
+      </c>
+      <c r="N40" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="O40" s="12" t="inlineStr">
+        <is>
+          <t>Unblock with TC-TRL-012 and access to the test mailbox.</t>
         </is>
       </c>
     </row>
@@ -4406,7 +5163,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="45" customHeight="1">
+    <row r="53" ht="72" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
           <t>5. Subscription Lifecycle and Premium Access</t>
@@ -4437,8 +5194,53 @@
           <t>Premium content is accessible.</t>
         </is>
       </c>
-    </row>
-    <row r="54" ht="45" customHeight="1">
+      <c r="G53" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H53" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I53" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J53" s="12" t="inlineStr">
+        <is>
+          <t>canceluser annual with ads, 15 EUR/year, active; deactiveaccount annual no ads, cancelled at trial end but still inside the period</t>
+        </is>
+      </c>
+      <c r="K53" s="12" t="inlineStr">
+        <is>
+          <t>4000056655665556; 2223003122003222</t>
+        </is>
+      </c>
+      <c r="L53" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M53" s="12" t="inlineStr">
+        <is>
+          <t>Both logins open /xtra/gestionar-suscripcion and see Tus beneficios Xtra. The logged-in article header CTA does not include is-visible. Stripe still shows canceluser as active: 15.00 EUR per year, next invoice 22 Oct 2027, Visa •••• 5556, Modo de prueba. deactiveaccount still sees the benefits list on 22 Oct 2026 while the cancelled trial period is open.</t>
+        </is>
+      </c>
+      <c r="N53" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/07-in-xtra.png; /tmp/section35/14-post-cancel-manage-now.png; /tmp/section35/15-post-cancel-article.png; /tmp/section35/24-canceluser-portal-now.png</t>
+        </is>
+      </c>
+      <c r="O53" s="12" t="inlineStr">
+        <is>
+          <t>The Xataka manage page also shows a cancellation banner for canceluser that Stripe does not confirm. Benefits remain available. See TC-LIF-006.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="72" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
           <t>5. Subscription Lifecycle and Premium Access</t>
@@ -4469,8 +5271,53 @@
           <t>Premium content is blocked or paywalled.</t>
         </is>
       </c>
-    </row>
-    <row r="55" ht="45" customHeight="1">
+      <c r="G54" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H54" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I54" s="12" t="inlineStr">
+        <is>
+          <t>Logged out (no Xataka session)</t>
+        </is>
+      </c>
+      <c r="J54" s="12" t="inlineStr">
+        <is>
+          <t>Not subscribed</t>
+        </is>
+      </c>
+      <c r="K54" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L54" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M54" s="12" t="inlineStr">
+        <is>
+          <t>A logged-out request to /xtra/gestionar-suscripcion redirects to https://testing.xataka.com/xtra and shows Elige tu plan. The article header CTA class is xtra-cta-hd-lead is-visible js-xtra-cta. The same article body stays readable logged out (about 16,872 characters, versus about 16,793 while logged in).</t>
+        </is>
+      </c>
+      <c r="N54" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/08-out-manage.png; /tmp/section35/20-anon-manage.png; /tmp/section35/03-out-article.png; /tmp/section35/21-anon-article.png</t>
+        </is>
+      </c>
+      <c r="O54" s="12" t="inlineStr">
+        <is>
+          <t>The subscriber area is gated. The sampled analysis article is not body-paywalled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="72" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
           <t>5. Subscription Lifecycle and Premium Access</t>
@@ -4501,8 +5348,53 @@
           <t>Subscription renews and active access continues.</t>
         </is>
       </c>
-    </row>
-    <row r="56" ht="45" customHeight="1">
+      <c r="G55" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H55" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I55" s="12" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J55" s="12" t="inlineStr">
+        <is>
+          <t>No active monthly subscription</t>
+        </is>
+      </c>
+      <c r="K55" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L55" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M55" s="12" t="inlineStr">
+        <is>
+          <t>Automatic monthly renewal was not triggered. No monthly Stripe subscription is active, and there is no Stripe test clock. An earlier plan change toward monthly returned Ha ocurrido un error y no se ha podido cambiar el plan.</t>
+        </is>
+      </c>
+      <c r="N55" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section2/33-after-plan-action.png</t>
+        </is>
+      </c>
+      <c r="O55" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: put a monthly test subscription on a Stripe test clock and advance it to the renewal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="72" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
           <t>5. Subscription Lifecycle and Premium Access</t>
@@ -4533,8 +5425,53 @@
           <t>Subscription renews and active access continues.</t>
         </is>
       </c>
-    </row>
-    <row r="57" ht="45" customHeight="1">
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H56" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I56" s="12" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J56" s="12" t="inlineStr">
+        <is>
+          <t>Annual with ads, 15 EUR/year, next invoice 22 Oct 2027</t>
+        </is>
+      </c>
+      <c r="K56" s="12" t="inlineStr">
+        <is>
+          <t>4000056655665556</t>
+        </is>
+      </c>
+      <c r="L56" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M56" s="12" t="inlineStr">
+        <is>
+          <t>canceluser has an active annual Stripe subscription. The portal says the next invoice date is 22 Oct 2027, and the last paid invoice is 22 Oct 2026 for 17.54 USD / 15.00 EUR. Renewal was not triggered. No Stripe test clock is available.</t>
+        </is>
+      </c>
+      <c r="N56" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/02-portal-canceluser.png; /tmp/section35/24-canceluser-portal-now.png</t>
+        </is>
+      </c>
+      <c r="O56" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: advance a Stripe test clock to 22 Oct 2027. Leave this subscription active. The Xataka page shows a cancellation banner that Stripe does not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="72" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
           <t>5. Subscription Lifecycle and Premium Access</t>
@@ -4565,8 +5502,53 @@
           <t>Retry logic applies and access state follows business rules for failed payments.</t>
         </is>
       </c>
-    </row>
-    <row r="58" ht="45" customHeight="1">
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H57" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I57" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J57" s="12" t="inlineStr">
+        <is>
+          <t>Not failed</t>
+        </is>
+      </c>
+      <c r="K57" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L57" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M57" s="12" t="inlineStr">
+        <is>
+          <t>A failed renewal was not triggered. Stripe test clock and Smart Retry access are not available, the same gap as TC-PAY-008.</t>
+        </is>
+      </c>
+      <c r="N57" s="12" t="inlineStr">
+        <is>
+          <t>TC-PAY-008</t>
+        </is>
+      </c>
+      <c r="O57" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: use a Stripe test clock with a declining renewal card, then record the access state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="72" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
           <t>5. Subscription Lifecycle and Premium Access</t>
@@ -4597,8 +5579,53 @@
           <t>Subscription is canceled according to configured cancellation timing.</t>
         </is>
       </c>
-    </row>
-    <row r="59" ht="45" customHeight="1">
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H58" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I58" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="J58" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, trial cancelled at period end</t>
+        </is>
+      </c>
+      <c r="K58" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="L58" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M58" s="12" t="inlineStr">
+        <is>
+          <t>User cancellation completed for deactiveaccount. Stripe shows Cancels Oct 22 and says the service will no longer be available after the free trial ends on October 22, 2026. Xataka shows Tu suscripción a Xtra está cancelada and No se renovará el 22 de octubre de 2026, while benefits remain until that date. Timing is the end of the current period.</t>
+        </is>
+      </c>
+      <c r="N58" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/10-cancelled.png; /tmp/section35/14-post-cancel-manage-now.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="O58" s="12" t="inlineStr">
+        <is>
+          <t>canceluser was not cancelled in Stripe. Its portal still shows Cancelar suscripción and next invoice 22 Oct 2027. The Xataka manage page for canceluser nevertheless says the subscription is cancelled and will not renew on 22 Oct 2026, and it offers Volver a activar tu suscripción. That banner does not match Stripe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="72" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
           <t>5. Subscription Lifecycle and Premium Access</t>
@@ -4629,8 +5656,53 @@
           <t>Premium access is removed when subscription is no longer active.</t>
         </is>
       </c>
-    </row>
-    <row r="60" ht="45" customHeight="1">
+      <c r="G59" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H59" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I59" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="J59" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, cancelled, effective 22 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K59" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="L59" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M59" s="12" t="inlineStr">
+        <is>
+          <t>On 22 Oct 2026, before the trial-end instant, deactiveaccount still opens Tus beneficios Xtra and the article header CTA stays hidden. Stripe says access ends after the free trial ends on October 22, 2026. Time could not be advanced past that instant, so removal of access after the effective date was not observed.</t>
+        </is>
+      </c>
+      <c r="N59" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/14-post-cancel-manage-now.png; /tmp/section35/15-post-cancel-article.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="O59" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: recheck after the trial end, or advance a Stripe test clock past 22 Oct 2026. Current benefits access is the in-period state, not the post-end state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="72" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
           <t>5. Subscription Lifecycle and Premium Access</t>
@@ -4661,8 +5733,53 @@
           <t>PayPal subscriber flow and premium access remain functional.</t>
         </is>
       </c>
-    </row>
-    <row r="61" ht="45" customHeight="1">
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H60" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I60" s="12" t="inlineStr">
+        <is>
+          <t>No PayPal subscriber in the working accounts</t>
+        </is>
+      </c>
+      <c r="J60" s="12" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="K60" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="L60" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M60" s="12" t="inlineStr">
+        <is>
+          <t>PayPal was not tested. Both working accounts are Stripe subscribers, Visa •••• 5556 and Mastercard •••• 3222. No known PayPal Xtra subscriber was available.</t>
+        </is>
+      </c>
+      <c r="N60" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/24-canceluser-portal-now.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="O60" s="12" t="inlineStr">
+        <is>
+          <t>Unblock: provide a PayPal Xtra subscriber on testing.xataka.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="72" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
           <t>5. Subscription Lifecycle and Premium Access</t>
@@ -4691,6 +5808,51 @@
       <c r="F61" s="2" t="inlineStr">
         <is>
           <t>New subscription is created through Stripe Billing.</t>
+        </is>
+      </c>
+      <c r="G61" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H61" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="I61" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="J61" s="12" t="inlineStr">
+        <is>
+          <t>Stripe trial on annual no ads; Stripe paid annual with ads</t>
+        </is>
+      </c>
+      <c r="K61" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222; 4000056655665556</t>
+        </is>
+      </c>
+      <c r="L61" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="M61" s="12" t="inlineStr">
+        <is>
+          <t>Both working subscriptions were created through Stripe in test mode. deactiveaccount has a Stripe trial with a 0.00 EUR trial invoice and a billing portal secret starting test_. canceluser has a Stripe paid subscription, invoice 17.54 USD, portal Modo de prueba, and the same test_ secret form. Checkout sessions used Stripe-hosted Checkout with cs_test_ session ids.</t>
+        </is>
+      </c>
+      <c r="N61" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/12-portal-after-cancel.png; /tmp/section35/24-canceluser-portal-now.png; TC-PAY-001 success URL cs_test_b184VAPjkmYPtr8CIq9XPdGE0q1ae2uEMWGm02PERdMaEdpcvzY1BJ9M8I</t>
+        </is>
+      </c>
+      <c r="O61" s="12" t="inlineStr">
+        <is>
+          <t>Production Checkout was not used. No live charge was submitted.</t>
         </is>
       </c>
     </row>
@@ -6418,7 +7580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11268,6 +12430,1556 @@
       <c r="L78" s="5" t="inlineStr">
         <is>
           <t>Homepage login panel was used. Shared password was used and is not stored in this workbook. XTRA was not opened because login was rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="60" customHeight="1">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-001</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E79" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F79" s="12" t="inlineStr">
+        <is>
+          <t>No 7-day plan. Catalog trial is 1 day.</t>
+        </is>
+      </c>
+      <c r="G79" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H79" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I79" s="12" t="inlineStr">
+        <is>
+          <t>Reviewed Stripe Checkout summaries already captured for monthly and both annual plans.</t>
+        </is>
+      </c>
+      <c r="J79" s="12" t="inlineStr">
+        <is>
+          <t>Checkout does not show a 7-day trial. Monthly Checkout showed 1 día gratis, then 2.34 USD per month. Both annual plans also showed a 1-day trial. A 7-day trial is not configured on testing.xataka.com.</t>
+        </is>
+      </c>
+      <c r="K79" s="12" t="inlineStr">
+        <is>
+          <t>TC-STR-003, TC-STR-009, TC-STR-010; /tmp/section2/05-stripe-or-blocker.png</t>
+        </is>
+      </c>
+      <c r="L79" s="12" t="inlineStr">
+        <is>
+          <t>Precondition absent. Do not treat the live 1-day trial as a 7-day configuration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="60" customHeight="1">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-002</t>
+        </is>
+      </c>
+      <c r="D80" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E80" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F80" s="12" t="inlineStr">
+        <is>
+          <t>No 14-day plan. Catalog trial is 1 day.</t>
+        </is>
+      </c>
+      <c r="G80" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H80" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I80" s="12" t="inlineStr">
+        <is>
+          <t>Compared the required 14-day duration with Checkout summaries from the testing catalog.</t>
+        </is>
+      </c>
+      <c r="J80" s="12" t="inlineStr">
+        <is>
+          <t>Checkout and subscription details do not show a 14-day trial. The testing catalog shows a 1-day trial on the monthly plan and on both annual plans.</t>
+        </is>
+      </c>
+      <c r="K80" s="12" t="inlineStr">
+        <is>
+          <t>TC-STR-009, TC-STR-010; /tmp/section2/05-stripe-or-blocker.png</t>
+        </is>
+      </c>
+      <c r="L80" s="12" t="inlineStr">
+        <is>
+          <t>Precondition absent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="60" customHeight="1">
+      <c r="A81" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C81" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-003</t>
+        </is>
+      </c>
+      <c r="D81" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E81" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F81" s="12" t="inlineStr">
+        <is>
+          <t>No 30-day plan. Catalog trial is 1 day.</t>
+        </is>
+      </c>
+      <c r="G81" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H81" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I81" s="12" t="inlineStr">
+        <is>
+          <t>Compared the required 30-day duration with Checkout summaries from the testing catalog.</t>
+        </is>
+      </c>
+      <c r="J81" s="12" t="inlineStr">
+        <is>
+          <t>Checkout and subscription details do not show a 30-day trial. The testing catalog shows a 1-day trial on the monthly plan and on both annual plans.</t>
+        </is>
+      </c>
+      <c r="K81" s="12" t="inlineStr">
+        <is>
+          <t>TC-STR-009, TC-STR-010; /tmp/section2/05-stripe-or-blocker.png</t>
+        </is>
+      </c>
+      <c r="L81" s="12" t="inlineStr">
+        <is>
+          <t>Precondition absent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="60" customHeight="1">
+      <c r="A82" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B82" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C82" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-004</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E82" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F82" s="12" t="inlineStr">
+        <is>
+          <t>Monthly 2 EUR; annual with ads 15 EUR; annual no ads 30 EUR. All showed 1 day.</t>
+        </is>
+      </c>
+      <c r="G82" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H82" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I82" s="12" t="inlineStr">
+        <is>
+          <t>Compared trial messaging across the three testing plans.</t>
+        </is>
+      </c>
+      <c r="J82" s="12" t="inlineStr">
+        <is>
+          <t>Monthly and both annual plans showed the same 1-day trial in Stripe Checkout. Distinct per-plan trial durations are not configured, so each plan using its own duration could not be compared.</t>
+        </is>
+      </c>
+      <c r="K82" s="12" t="inlineStr">
+        <is>
+          <t>TC-STR-010; /tmp/section2/05-stripe-or-blocker.png</t>
+        </is>
+      </c>
+      <c r="L82" s="12" t="inlineStr">
+        <is>
+          <t>Precondition of different trial settings is not met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="60" customHeight="1">
+      <c r="A83" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C83" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-005</t>
+        </is>
+      </c>
+      <c r="D83" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E83" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="F83" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, 1-day trial</t>
+        </is>
+      </c>
+      <c r="G83" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222 (already on the trial; not re-entered)</t>
+        </is>
+      </c>
+      <c r="H83" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I83" s="12" t="inlineStr">
+        <is>
+          <t>Logged in from the testing homepage, opened the subscriber area and an article while the trial was active.</t>
+        </is>
+      </c>
+      <c r="J83" s="12" t="inlineStr">
+        <is>
+          <t>deactiveaccount opened /xtra/gestionar-suscripcion during the trial and saw Tus beneficios Xtra, including Discord, consultorio, sorteos, and newsletters. On an article, the header CTA class was xtra-cta-hd-lead js-xtra-cta and did not include is-visible.</t>
+        </is>
+      </c>
+      <c r="K83" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/01-deactive-manage.png; /tmp/section35/05-in-article.png; /tmp/section35/06-in-sorteo.png; /tmp/section35/07-in-xtra.png</t>
+        </is>
+      </c>
+      <c r="L83" s="12" t="inlineStr">
+        <is>
+          <t>Trial access was already active before this cancellation run. Individual Discord and live-event destinations were not each opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="60" customHeight="1">
+      <c r="A84" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B84" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C84" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-006</t>
+        </is>
+      </c>
+      <c r="D84" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E84" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="F84" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, 1-day trial</t>
+        </is>
+      </c>
+      <c r="G84" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="H84" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I84" s="12" t="inlineStr">
+        <is>
+          <t>Opened the Stripe Customer Portal for the trial subscription and read invoice history.</t>
+        </is>
+      </c>
+      <c r="J84" s="12" t="inlineStr">
+        <is>
+          <t>The only Stripe invoice during the trial is 21 Oct 2026, 0.00 EUR, Paid, description Trial period for Xataka Xtra. No charge was generated. The portal lists Mastercard •••• 3222.</t>
+        </is>
+      </c>
+      <c r="K84" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/02-portal-deactive.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="L84" s="12" t="inlineStr">
+        <is>
+          <t>No charge before the trial end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="60" customHeight="1">
+      <c r="A85" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B85" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C85" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-007</t>
+        </is>
+      </c>
+      <c r="D85" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E85" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="F85" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, 1-day trial</t>
+        </is>
+      </c>
+      <c r="G85" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="H85" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I85" s="12" t="inlineStr">
+        <is>
+          <t>Compared the Xataka renewal date with the Stripe trial-end date.</t>
+        </is>
+      </c>
+      <c r="J85" s="12" t="inlineStr">
+        <is>
+          <t>Before cancellation, the Xataka subscription page said the plan would renew on 22 Oct 2026 for 30 EUR/year. Stripe said the free trial ends Oct 22. After cancellation, Stripe says the service will no longer be available after the free trial ends on October 22, 2026. The date matches the trial end.</t>
+        </is>
+      </c>
+      <c r="K85" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/01-deactive-manage.png; /tmp/section35/02-portal-deactive.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="L85" s="12" t="inlineStr">
+        <is>
+          <t>Match is 22 Oct 2026 on both sides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="60" customHeight="1">
+      <c r="A86" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B86" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C86" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-008</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E86" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F86" s="12" t="inlineStr">
+        <is>
+          <t>deactiveaccount trial cancelled before the end; canceluser is already a paid annual plan</t>
+        </is>
+      </c>
+      <c r="G86" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H86" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I86" s="12" t="inlineStr">
+        <is>
+          <t>Checked both subscriptions for a trial that reached its end without cancellation.</t>
+        </is>
+      </c>
+      <c r="J86" s="12" t="inlineStr">
+        <is>
+          <t>Automatic conversion at trial end was not observed. The deactiveaccount trial was cancelled before the end. canceluser's 22 Oct 2026 invoice for 17.54 USD was an immediate charge with no trial, not a trial conversion. No Stripe test clock is available.</t>
+        </is>
+      </c>
+      <c r="K86" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/12-portal-after-cancel.png; /tmp/section35/24-canceluser-portal-now.png</t>
+        </is>
+      </c>
+      <c r="L86" s="12" t="inlineStr">
+        <is>
+          <t>Conversion was not triggered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="60" customHeight="1">
+      <c r="A87" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C87" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-009</t>
+        </is>
+      </c>
+      <c r="D87" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E87" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="F87" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, 1-day trial</t>
+        </is>
+      </c>
+      <c r="G87" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="H87" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I87" s="12" t="inlineStr">
+        <is>
+          <t>Logged in as deactiveaccount, opened cancel subscription, selected a reason, and confirmed. Then reopened the Stripe portal.</t>
+        </is>
+      </c>
+      <c r="J87" s="12" t="inlineStr">
+        <is>
+          <t>Cancelled the trial from /xtra/gestionar-suscripcion/cancelar-suscripcion after choosing Otra razón. Confirmation said Suscripción cancelada con éxito, and that Xtra continues until 22 Oct 2026 and will not renew. Stripe test portal shows Cancels Oct 22, 30.00 EUR per year, and says the service will no longer be available after the free trial ends. Invoice history is still only the 0.00 EUR trial invoice.</t>
+        </is>
+      </c>
+      <c r="K87" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/09-cancel-dialog.png; /tmp/section35/10-cancelled.png; /tmp/section35/11-after-cancel-manage.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="L87" s="12" t="inlineStr">
+        <is>
+          <t>No paid invoice was created by the cancellation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="60" customHeight="1">
+      <c r="A88" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B88" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C88" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-010</t>
+        </is>
+      </c>
+      <c r="D88" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E88" s="12" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser); follow-up on testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="F88" s="12" t="inlineStr">
+        <is>
+          <t>Annual with ads, 15 EUR/year, on the second checkout</t>
+        </is>
+      </c>
+      <c r="G88" s="12" t="inlineStr">
+        <is>
+          <t>4000056655665556 (card already stored on the paid subscription)</t>
+        </is>
+      </c>
+      <c r="H88" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I88" s="12" t="inlineStr">
+        <is>
+          <t>Read the prior second Checkout for canceluser. Clicked Suscríbete ahora while deactiveaccount's cancelled trial was still open and stopped when Checkout did not open.</t>
+        </is>
+      </c>
+      <c r="J88" s="12" t="inlineStr">
+        <is>
+          <t>A later Stripe Checkout for canceluser, after a trial had already been used, showed Suscribirse a Xataka Xtra, Total a pagar hoy 17.54 USD, and no 1 día gratis line. The paid invoice is 22 Oct 2026 for 17.54 USD / 15.00 EUR. In this run, Suscríbete ahora for deactiveaccount returned to /xtra/gestionar-suscripcion while the cancelled trial is still open, and did not open another trial checkout. No payment was submitted in this run.</t>
+        </is>
+      </c>
+      <c r="K88" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section2/results.json (second checkout text); /tmp/section35/02-portal-canceluser.png; /tmp/section35/17-after-subscribe-click.png; /tmp/section35/24-canceluser-portal-now.png</t>
+        </is>
+      </c>
+      <c r="L88" s="12" t="inlineStr">
+        <is>
+          <t>One trial per account is supported by the immediate charge on the second checkout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="60" customHeight="1">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C89" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-011</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E89" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F89" s="12" t="inlineStr">
+        <is>
+          <t>Not changed</t>
+        </is>
+      </c>
+      <c r="G89" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H89" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I89" s="12" t="inlineStr">
+        <is>
+          <t>Confirmed Dar de baja is present and left it unused.</t>
+        </is>
+      </c>
+      <c r="J89" s="12" t="inlineStr">
+        <is>
+          <t>Account deactivation and reactivation were not performed. The account menu shows Dar de baja, and that control was not used. The 10 newly supplied emails cannot log in, so there is no reactivated account to test.</t>
+        </is>
+      </c>
+      <c r="K89" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/13-post-home-login.png</t>
+        </is>
+      </c>
+      <c r="L89" s="12" t="inlineStr">
+        <is>
+          <t>Do not deactivate the remaining paid fixture without a spare account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="60" customHeight="1">
+      <c r="A90" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B90" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C90" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-012</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E90" s="12" t="inlineStr">
+        <is>
+          <t>No second fresh account. 10 supplied emails are rejected at login.</t>
+        </is>
+      </c>
+      <c r="F90" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G90" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H90" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I90" s="12" t="inlineStr">
+        <is>
+          <t>Did not submit a card from a second account.</t>
+        </is>
+      </c>
+      <c r="J90" s="12" t="inlineStr">
+        <is>
+          <t>A duplicate trial with the same card fingerprint from another account was not executed. The 10 supplied emails cannot log in, and a new trial was not submitted from the two working accounts.</t>
+        </is>
+      </c>
+      <c r="K90" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="L90" s="12" t="inlineStr">
+        <is>
+          <t>Fingerprint, refund, error page, activation, and welcome mail all depend on this path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="60" customHeight="1">
+      <c r="A91" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B91" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C91" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-013</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E91" s="12" t="inlineStr">
+        <is>
+          <t>Depends on TC-TRL-012</t>
+        </is>
+      </c>
+      <c r="F91" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G91" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H91" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I91" s="12" t="inlineStr">
+        <is>
+          <t>Not run. No duplicate charge exists.</t>
+        </is>
+      </c>
+      <c r="J91" s="12" t="inlineStr">
+        <is>
+          <t>No duplicate-trial charge was created, so a refund could not be observed.</t>
+        </is>
+      </c>
+      <c r="K91" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="L91" s="12" t="inlineStr">
+        <is>
+          <t>Blocked on the missing second account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="60" customHeight="1">
+      <c r="A92" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B92" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C92" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-014</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E92" s="12" t="inlineStr">
+        <is>
+          <t>Depends on TC-TRL-012</t>
+        </is>
+      </c>
+      <c r="F92" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G92" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H92" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I92" s="12" t="inlineStr">
+        <is>
+          <t>Not run. Duplicate detection was not triggered.</t>
+        </is>
+      </c>
+      <c r="J92" s="12" t="inlineStr">
+        <is>
+          <t>The post-Checkout error page for a card already used on a free trial was not reached.</t>
+        </is>
+      </c>
+      <c r="K92" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="L92" s="12" t="inlineStr">
+        <is>
+          <t>Blocked on the missing second account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="60" customHeight="1">
+      <c r="A93" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B93" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C93" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-015</t>
+        </is>
+      </c>
+      <c r="D93" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E93" s="12" t="inlineStr">
+        <is>
+          <t>Depends on TC-TRL-012</t>
+        </is>
+      </c>
+      <c r="F93" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G93" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H93" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I93" s="12" t="inlineStr">
+        <is>
+          <t>Not run.</t>
+        </is>
+      </c>
+      <c r="J93" s="12" t="inlineStr">
+        <is>
+          <t>Subscription activation after duplicate-trial detection was not observed because the duplicate path was not started.</t>
+        </is>
+      </c>
+      <c r="K93" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="L93" s="12" t="inlineStr">
+        <is>
+          <t>Blocked on the missing second account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="60" customHeight="1">
+      <c r="A94" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B94" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C94" s="12" t="inlineStr">
+        <is>
+          <t>TC-TRL-016</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E94" s="12" t="inlineStr">
+        <is>
+          <t>Depends on TC-TRL-012</t>
+        </is>
+      </c>
+      <c r="F94" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G94" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H94" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I94" s="12" t="inlineStr">
+        <is>
+          <t>Not run.</t>
+        </is>
+      </c>
+      <c r="J94" s="12" t="inlineStr">
+        <is>
+          <t>Welcome screens and welcome email for a duplicate trial were not observed. The duplicate path was not started, and the mailbox was not inspected.</t>
+        </is>
+      </c>
+      <c r="K94" s="12" t="inlineStr">
+        <is>
+          <t>QA Accounts sheet, RUN-STR-20261022-007</t>
+        </is>
+      </c>
+      <c r="L94" s="12" t="inlineStr">
+        <is>
+          <t>Blocked on the missing second account and mailbox access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="60" customHeight="1">
+      <c r="A95" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B95" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C95" s="12" t="inlineStr">
+        <is>
+          <t>TC-LIF-001</t>
+        </is>
+      </c>
+      <c r="D95" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E95" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F95" s="12" t="inlineStr">
+        <is>
+          <t>canceluser annual with ads, 15 EUR/year, active; deactiveaccount annual no ads, cancelled at trial end but still inside the period</t>
+        </is>
+      </c>
+      <c r="G95" s="12" t="inlineStr">
+        <is>
+          <t>4000056655665556; 2223003122003222</t>
+        </is>
+      </c>
+      <c r="H95" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I95" s="12" t="inlineStr">
+        <is>
+          <t>Logged in from the homepage for each account, opened the subscriber area, and compared canceluser with the Stripe portal.</t>
+        </is>
+      </c>
+      <c r="J95" s="12" t="inlineStr">
+        <is>
+          <t>Both logins open /xtra/gestionar-suscripcion and see Tus beneficios Xtra. The logged-in article header CTA does not include is-visible. Stripe still shows canceluser as active: 15.00 EUR per year, next invoice 22 Oct 2027, Visa •••• 5556, Modo de prueba. deactiveaccount still sees the benefits list on 22 Oct 2026 while the cancelled trial period is open.</t>
+        </is>
+      </c>
+      <c r="K95" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/07-in-xtra.png; /tmp/section35/14-post-cancel-manage-now.png; /tmp/section35/15-post-cancel-article.png; /tmp/section35/24-canceluser-portal-now.png</t>
+        </is>
+      </c>
+      <c r="L95" s="12" t="inlineStr">
+        <is>
+          <t>Premium subscriber area is accessible for the active paid subscription.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="60" customHeight="1">
+      <c r="A96" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B96" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C96" s="12" t="inlineStr">
+        <is>
+          <t>TC-LIF-002</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E96" s="12" t="inlineStr">
+        <is>
+          <t>Logged out (no Xataka session)</t>
+        </is>
+      </c>
+      <c r="F96" s="12" t="inlineStr">
+        <is>
+          <t>Not subscribed</t>
+        </is>
+      </c>
+      <c r="G96" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H96" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I96" s="12" t="inlineStr">
+        <is>
+          <t>Opened the subscriber URL and the same article in a fresh browser context with no login.</t>
+        </is>
+      </c>
+      <c r="J96" s="12" t="inlineStr">
+        <is>
+          <t>A logged-out request to /xtra/gestionar-suscripcion redirects to https://testing.xataka.com/xtra and shows Elige tu plan. The article header CTA class is xtra-cta-hd-lead is-visible js-xtra-cta. The same article body stays readable logged out (about 16,872 characters, versus about 16,793 while logged in).</t>
+        </is>
+      </c>
+      <c r="K96" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/08-out-manage.png; /tmp/section35/20-anon-manage.png; /tmp/section35/03-out-article.png; /tmp/section35/21-anon-article.png</t>
+        </is>
+      </c>
+      <c r="L96" s="12" t="inlineStr">
+        <is>
+          <t>Partial because premium gating is the subscriber area and header CTA, not the article body.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="60" customHeight="1">
+      <c r="A97" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B97" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C97" s="12" t="inlineStr">
+        <is>
+          <t>TC-LIF-003</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E97" s="12" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F97" s="12" t="inlineStr">
+        <is>
+          <t>No active monthly subscription</t>
+        </is>
+      </c>
+      <c r="G97" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H97" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I97" s="12" t="inlineStr">
+        <is>
+          <t>Confirmed there is no monthly subscription to renew.</t>
+        </is>
+      </c>
+      <c r="J97" s="12" t="inlineStr">
+        <is>
+          <t>Automatic monthly renewal was not triggered. No monthly Stripe subscription is active, and there is no Stripe test clock. An earlier plan change toward monthly returned Ha ocurrido un error y no se ha podido cambiar el plan.</t>
+        </is>
+      </c>
+      <c r="K97" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section2/33-after-plan-action.png</t>
+        </is>
+      </c>
+      <c r="L97" s="12" t="inlineStr">
+        <is>
+          <t>Blocked on plan state and missing test clock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="60" customHeight="1">
+      <c r="A98" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B98" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C98" s="12" t="inlineStr">
+        <is>
+          <t>TC-LIF-004</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E98" s="12" t="inlineStr">
+        <is>
+          <t>testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F98" s="12" t="inlineStr">
+        <is>
+          <t>Annual with ads, 15 EUR/year, next invoice 22 Oct 2027</t>
+        </is>
+      </c>
+      <c r="G98" s="12" t="inlineStr">
+        <is>
+          <t>4000056655665556</t>
+        </is>
+      </c>
+      <c r="H98" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I98" s="12" t="inlineStr">
+        <is>
+          <t>Opened the Stripe Customer Portal and read the next invoice date. Did not click Cancelar suscripción.</t>
+        </is>
+      </c>
+      <c r="J98" s="12" t="inlineStr">
+        <is>
+          <t>canceluser has an active annual Stripe subscription. The portal says the next invoice date is 22 Oct 2027, and the last paid invoice is 22 Oct 2026 for 17.54 USD / 15.00 EUR. Renewal was not triggered. No Stripe test clock is available.</t>
+        </is>
+      </c>
+      <c r="K98" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/02-portal-canceluser.png; /tmp/section35/24-canceluser-portal-now.png</t>
+        </is>
+      </c>
+      <c r="L98" s="12" t="inlineStr">
+        <is>
+          <t>Renewal date is one year out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="60" customHeight="1">
+      <c r="A99" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C99" s="12" t="inlineStr">
+        <is>
+          <t>TC-LIF-005</t>
+        </is>
+      </c>
+      <c r="D99" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E99" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F99" s="12" t="inlineStr">
+        <is>
+          <t>Not failed</t>
+        </is>
+      </c>
+      <c r="G99" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H99" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I99" s="12" t="inlineStr">
+        <is>
+          <t>Not run. No failed renewal was created.</t>
+        </is>
+      </c>
+      <c r="J99" s="12" t="inlineStr">
+        <is>
+          <t>A failed renewal was not triggered. Stripe test clock and Smart Retry access are not available, the same gap as TC-PAY-008.</t>
+        </is>
+      </c>
+      <c r="K99" s="12" t="inlineStr">
+        <is>
+          <t>TC-PAY-008</t>
+        </is>
+      </c>
+      <c r="L99" s="12" t="inlineStr">
+        <is>
+          <t>Blocked on missing test clock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="60" customHeight="1">
+      <c r="A100" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B100" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C100" s="12" t="inlineStr">
+        <is>
+          <t>TC-LIF-006</t>
+        </is>
+      </c>
+      <c r="D100" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E100" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="F100" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, 30 EUR/year, trial cancelled at period end</t>
+        </is>
+      </c>
+      <c r="G100" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="H100" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I100" s="12" t="inlineStr">
+        <is>
+          <t>Cancelled deactiveaccount at period end. Re-read both manage pages and the canceluser Stripe portal without clicking cancel or reactivate.</t>
+        </is>
+      </c>
+      <c r="J100" s="12" t="inlineStr">
+        <is>
+          <t>User cancellation completed for deactiveaccount. Stripe shows Cancels Oct 22 and says the service will no longer be available after the free trial ends on October 22, 2026. Xataka shows Tu suscripción a Xtra está cancelada and No se renovará el 22 de octubre de 2026, while benefits remain until that date. Timing is the end of the current period.</t>
+        </is>
+      </c>
+      <c r="K100" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/10-cancelled.png; /tmp/section35/14-post-cancel-manage-now.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="L100" s="12" t="inlineStr">
+        <is>
+          <t>Executed cancellation matches Stripe for deactiveaccount. The paid account's Xataka banner is a mismatch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="60" customHeight="1">
+      <c r="A101" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B101" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C101" s="12" t="inlineStr">
+        <is>
+          <t>TC-LIF-007</t>
+        </is>
+      </c>
+      <c r="D101" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E101" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount)</t>
+        </is>
+      </c>
+      <c r="F101" s="12" t="inlineStr">
+        <is>
+          <t>Annual no ads, cancelled, effective 22 Oct 2026</t>
+        </is>
+      </c>
+      <c r="G101" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222</t>
+        </is>
+      </c>
+      <c r="H101" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I101" s="12" t="inlineStr">
+        <is>
+          <t>Rechecked the subscriber area and an article on the cancellation end date.</t>
+        </is>
+      </c>
+      <c r="J101" s="12" t="inlineStr">
+        <is>
+          <t>On 22 Oct 2026, before the trial-end instant, deactiveaccount still opens Tus beneficios Xtra and the article header CTA stays hidden. Stripe says access ends after the free trial ends on October 22, 2026. Time could not be advanced past that instant, so removal of access after the effective date was not observed.</t>
+        </is>
+      </c>
+      <c r="K101" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/14-post-cancel-manage-now.png; /tmp/section35/15-post-cancel-article.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="L101" s="12" t="inlineStr">
+        <is>
+          <t>Effective instant has not passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="60" customHeight="1">
+      <c r="A102" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B102" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C102" s="12" t="inlineStr">
+        <is>
+          <t>TC-LIF-008</t>
+        </is>
+      </c>
+      <c r="D102" s="11" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E102" s="12" t="inlineStr">
+        <is>
+          <t>No PayPal subscriber in the working accounts</t>
+        </is>
+      </c>
+      <c r="F102" s="12" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="G102" s="12" t="inlineStr">
+        <is>
+          <t>No new card submitted</t>
+        </is>
+      </c>
+      <c r="H102" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I102" s="12" t="inlineStr">
+        <is>
+          <t>Confirmed the stored payment methods are cards.</t>
+        </is>
+      </c>
+      <c r="J102" s="12" t="inlineStr">
+        <is>
+          <t>PayPal was not tested. Both working accounts are Stripe subscribers, Visa •••• 5556 and Mastercard •••• 3222. No known PayPal Xtra subscriber was available.</t>
+        </is>
+      </c>
+      <c r="K102" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/24-canceluser-portal-now.png; /tmp/section35/12-portal-after-cancel.png</t>
+        </is>
+      </c>
+      <c r="L102" s="12" t="inlineStr">
+        <is>
+          <t>PayPal coexistence was not exercised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="60" customHeight="1">
+      <c r="A103" s="12" t="inlineStr">
+        <is>
+          <t>RUN-STR-20261022-008</t>
+        </is>
+      </c>
+      <c r="B103" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:29 UTC</t>
+        </is>
+      </c>
+      <c r="C103" s="12" t="inlineStr">
+        <is>
+          <t>TC-LIF-009</t>
+        </is>
+      </c>
+      <c r="D103" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E103" s="12" t="inlineStr">
+        <is>
+          <t>testi.n.g.2.4.aug@gmail.com (username deactiveaccount); testing24au.g2.6@gmail.com (username canceluser)</t>
+        </is>
+      </c>
+      <c r="F103" s="12" t="inlineStr">
+        <is>
+          <t>Stripe trial on annual no ads; Stripe paid annual with ads</t>
+        </is>
+      </c>
+      <c r="G103" s="12" t="inlineStr">
+        <is>
+          <t>2223003122003222; 4000056655665556</t>
+        </is>
+      </c>
+      <c r="H103" s="12" t="inlineStr">
+        <is>
+          <t>Testing - testing.xataka.com; Stripe test mode (Modo de prueba, billing portal secret=test_)</t>
+        </is>
+      </c>
+      <c r="I103" s="12" t="inlineStr">
+        <is>
+          <t>Confirmed both Customer Portal sessions are Stripe test-mode sessions.</t>
+        </is>
+      </c>
+      <c r="J103" s="12" t="inlineStr">
+        <is>
+          <t>Both working subscriptions were created through Stripe in test mode. deactiveaccount has a Stripe trial with a 0.00 EUR trial invoice and a billing portal secret starting test_. canceluser has a Stripe paid subscription, invoice 17.54 USD, portal Modo de prueba, and the same test_ secret form. Checkout sessions used Stripe-hosted Checkout with cs_test_ session ids.</t>
+        </is>
+      </c>
+      <c r="K103" s="12" t="inlineStr">
+        <is>
+          <t>/tmp/section35/12-portal-after-cancel.png; /tmp/section35/24-canceluser-portal-now.png; TC-PAY-001 success URL cs_test_b184VAPjkmYPtr8CIq9XPdGE0q1ae2uEMWGm02PERdMaEdpcvzY1BJ9M8I</t>
+        </is>
+      </c>
+      <c r="L103" s="12" t="inlineStr">
+        <is>
+          <t>New subscriptions observed in this environment are Stripe Billing subscriptions.</t>
         </is>
       </c>
     </row>

</xml_diff>